<commit_message>
📊 Horarios actualizados Línea 141 - 4575
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:02:18</t>
+          <t>Última actualización: 00:49:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -473,12 +473,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>00:02:18</t>
+          <t>00:49:31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>01:13</t>
+          <t>01:12</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -487,7 +487,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>71</v>
+        <v>23</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -503,18 +503,68 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>01:13</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>71</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>00:49:31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>01:58</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>69</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>00:02:18</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>01:59</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D7" t="n">
+      <c r="D9" t="n">
         <v>117</v>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -531,7 +581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,14 +594,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:02:18</t>
+          <t>Última actualización: 00:49:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -585,23 +635,48 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>00:49:31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>01:12</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>23</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>00:02:18</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>01:13</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D6" t="n">
+      <c r="D7" t="n">
         <v>71</v>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -631,7 +706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:02:18</t>
+          <t>Última actualización: 00:49:31</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4576
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:31</t>
+          <t>Última actualización: 01:17:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>00:02:18</t>
+          <t>01:17:21</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -562,9 +562,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>117</v>
+        <v>42</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>01:17:21</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>02:57</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>100</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -581,7 +606,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,14 +619,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:31</t>
+          <t>Última actualización: 01:17:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 3</t>
         </is>
       </c>
     </row>
@@ -677,6 +702,31 @@
         <v>71</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>01:17:21</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>02:57</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>100</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -706,7 +756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 00:49:31</t>
+          <t>Última actualización: 01:17:21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4577
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:17:21</t>
+          <t>Última actualización: 01:51:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -523,7 +523,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>00:49:31</t>
+          <t>01:51:30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -537,7 +537,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -573,23 +573,98 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>01:51:30</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>65</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>01:17:21</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>02:57</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>100</v>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>01:51:30</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>03:01</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>70</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>01:51:30</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>03:48</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>117</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -606,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -619,14 +694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:17:21</t>
+          <t>Última actualización: 01:51:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 3</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -710,23 +785,48 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>01:51:30</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>02:56</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>65</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>01:17:21</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>02:57</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>215_ALUAR</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>100</v>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -756,7 +856,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:17:21</t>
+          <t>Última actualización: 01:51:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4578
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:51:30</t>
+          <t>Última actualización: 02:16:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>01:17:21</t>
+          <t>02:16:13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>01:51:30</t>
+          <t>02:16:13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,9 +662,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>117</v>
+        <v>92</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>02:16:13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>96</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -681,7 +706,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -694,14 +719,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:51:30</t>
+          <t>Última actualización: 02:16:13</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 5</t>
         </is>
       </c>
     </row>
@@ -810,7 +835,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>01:17:21</t>
+          <t>02:16:13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -824,9 +849,34 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>02:16:13</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>03:52</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215_ALUAR</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>96</v>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -856,7 +906,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 01:51:30</t>
+          <t>Última actualización: 02:16:13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4579
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:13</t>
+          <t>Última actualización: 02:43:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>02:16:13</t>
+          <t>02:43:20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -612,7 +612,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>02:16:13</t>
+          <t>02:43:20</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>02:16:13</t>
+          <t>02:43:20</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,9 +687,34 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>02:43:20</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>04:32</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>109</v>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -719,7 +744,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:13</t>
+          <t>Última actualización: 02:43:20</t>
         </is>
       </c>
     </row>
@@ -835,7 +860,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>02:16:13</t>
+          <t>02:43:20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -849,7 +874,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -860,7 +885,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:16:13</t>
+          <t>02:43:20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -874,7 +899,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -906,7 +931,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:16:13</t>
+          <t>Última actualización: 02:43:20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4580
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:43:20</t>
+          <t>Última actualización: 03:01:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -648,7 +648,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>02:43:20</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>02:43:20</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -687,7 +687,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -698,7 +698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>02:43:20</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -712,9 +712,59 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>03:01:03</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>104</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>03:01:03</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>107</v>
+      </c>
+      <c r="E17" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -731,7 +781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -744,14 +794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:43:20</t>
+          <t>Última actualización: 03:01:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -885,7 +935,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>02:43:20</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -899,9 +949,34 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>03:01:03</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>107</v>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -931,7 +1006,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 02:43:20</t>
+          <t>Última actualización: 03:01:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4581
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:01:03</t>
+          <t>Última actualización: 03:54:03</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -698,21 +698,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>04:32</t>
+          <t>04:02</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>91</v>
+        <v>8</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -728,16 +728,16 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>04:32</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -753,18 +753,193 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>104</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>04:48</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>54</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>03:01:03</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D17" t="n">
+      <c r="D19" t="n">
         <v>107</v>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>04:53</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>59</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>05:17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>83</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>05:22</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>88</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>110</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>03:54:03</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>05:47</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>113</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -794,7 +969,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:01:03</t>
+          <t>Última actualización: 03:54:03</t>
         </is>
       </c>
     </row>
@@ -1006,7 +1181,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:01:03</t>
+          <t>Última actualización: 03:54:03</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4582
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:54:03</t>
+          <t>Última actualización: 04:21:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -773,12 +773,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>04:21:29</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>04:48</t>
+          <t>04:47</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -787,7 +787,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>54</v>
+        <v>26</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,21 +823,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>04:53</t>
+          <t>04:48</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>59</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -848,21 +848,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>04:21:29</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>05:17</t>
+          <t>04:53</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,21 +873,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>04:21:29</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>05:22</t>
+          <t>05:17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>88</v>
+        <v>56</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,21 +898,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>04:21:29</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>05:44</t>
+          <t>05:22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>110</v>
+        <v>61</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -923,23 +923,148 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>05:40</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>79</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>03:54:03</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>110</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>05:47</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>113</v>
-      </c>
-      <c r="E24" t="inlineStr">
+      <c r="D26" t="n">
+        <v>86</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>06:01</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>100</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>06:09</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>108</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>111</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -956,7 +1081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -969,14 +1094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:54:03</t>
+          <t>Última actualización: 04:21:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 7</t>
         </is>
       </c>
     </row>
@@ -1152,6 +1277,31 @@
         <v>107</v>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>04:21:29</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>06:12</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>111</v>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1181,7 +1331,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 03:54:03</t>
+          <t>Última actualización: 04:21:29</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4583
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:21:29</t>
+          <t>Última actualización: 04:51:30</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -848,7 +848,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>32</v>
+        <v>2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>56</v>
+        <v>26</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>61</v>
+        <v>31</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>110</v>
+        <v>53</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>86</v>
+        <v>56</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>108</v>
+        <v>78</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,9 +1062,134 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>04:51:30</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>06:30</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>99</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>04:51:30</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>06:34</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>103</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>04:51:30</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>108</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>04:51:30</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>06:39</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>108</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>04:51:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>06:41</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>110</v>
+      </c>
+      <c r="E34" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1094,7 +1219,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:21:29</t>
+          <t>Última actualización: 04:51:30</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1410,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:21:29</t>
+          <t>04:51:30</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1299,7 +1424,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1331,7 +1456,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:21:29</t>
+          <t>Última actualización: 04:51:30</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4584
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:30</t>
+          <t>Última actualización: 05:15:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -873,7 +873,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -887,7 +887,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>31</v>
+        <v>7</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -948,7 +948,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -962,7 +962,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1012,7 +1012,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>70</v>
+        <v>46</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>78</v>
+        <v>54</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>103</v>
+        <v>79</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>108</v>
+        <v>84</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,7 +1173,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1187,9 +1187,59 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>05:15:08</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>100</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>05:15:08</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>06:59</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>104</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1206,7 +1256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1219,14 +1269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:30</t>
+          <t>Última actualización: 05:15:08</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 7</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1410,7 +1460,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>04:51:30</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1424,9 +1474,34 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>81</v>
+        <v>57</v>
       </c>
       <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05:15:08</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1456,7 +1531,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 04:51:30</t>
+          <t>Última actualización: 05:15:08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4585
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:08</t>
+          <t>Última actualización: 05:47:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1023,7 +1023,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1037,7 +1037,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>54</v>
+        <v>22</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1048,7 +1048,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1062,7 +1062,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,7 +1073,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>75</v>
+        <v>43</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,7 +1098,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1112,7 +1112,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>79</v>
+        <v>47</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,7 +1123,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1133,11 +1133,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1158,11 +1158,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>84</v>
+        <v>52</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,12 +1173,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1187,7 +1187,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>86</v>
+        <v>53</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1203,16 +1203,16 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,23 +1223,198 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>06:55</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>68</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>06:59</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>104</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>72</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>92</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>92</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>93</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>108</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>109</v>
+      </c>
+      <c r="E43" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1256,7 +1431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1269,14 +1444,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:08</t>
+          <t>Última actualización: 05:47:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1635,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1474,7 +1649,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>57</v>
+        <v>25</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1485,7 +1660,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>05:47:42</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1499,9 +1674,34 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>100</v>
+        <v>68</v>
       </c>
       <c r="E13" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>07:19</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>92</v>
+      </c>
+      <c r="E14" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1518,7 +1718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1531,14 +1731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:15:08</t>
+          <t>Última actualización: 05:47:42</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 1</t>
+          <t>Total filas: 2</t>
         </is>
       </c>
     </row>
@@ -1589,6 +1789,31 @@
         <v>15</v>
       </c>
       <c r="E6" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>05:47:42</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>07:43</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>116</v>
+      </c>
+      <c r="E7" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4586
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:47:42</t>
+          <t>Última actualización: 06:10:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -1048,21 +1048,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>06:12</t>
+          <t>06:10</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -1073,21 +1073,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>06:30</t>
+          <t>06:12</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1098,21 +1098,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>06:34</t>
+          <t>06:30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1123,21 +1123,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>06:39</t>
+          <t>06:34</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -1148,7 +1148,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>52</v>
+        <v>29</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1173,21 +1173,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>06:40</t>
+          <t>06:39</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1198,12 +1198,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>05:15:08</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>06:41</t>
+          <t>06:40</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1223,21 +1223,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>05:15:08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:41</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>68</v>
+        <v>86</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1273,21 +1273,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1308,11 +1308,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>93</v>
+        <v>69</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>108</v>
+        <v>76</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,23 +1398,98 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>85</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>06:10:41</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>07:36</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D43" t="n">
+      <c r="D44" t="n">
+        <v>86</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>06:10:41</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>105</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>06:10:41</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>07:59</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
         <v>109</v>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1444,7 +1519,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:47:42</t>
+          <t>Última actualización: 06:10:41</t>
         </is>
       </c>
     </row>
@@ -1635,7 +1710,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1649,7 +1724,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>25</v>
+        <v>2</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -1660,7 +1735,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1674,7 +1749,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1685,7 +1760,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1699,7 +1774,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -1731,7 +1806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 05:47:42</t>
+          <t>Última actualización: 06:10:41</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1872,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>05:47:42</t>
+          <t>06:10:41</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1811,7 +1886,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>116</v>
+        <v>93</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4587
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:10:41</t>
+          <t>Última actualización: 06:43:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1248,21 +1248,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>06:55</t>
+          <t>06:43</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -1278,16 +1278,16 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>06:59</t>
+          <t>06:55</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1298,21 +1298,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:56</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>69</v>
+        <v>13</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1323,21 +1323,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>06:59</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1353,16 +1353,16 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,21 +1373,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>76</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1403,16 +1403,16 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,21 +1423,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>86</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,21 +1448,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>105</v>
+        <v>38</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1478,18 +1478,368 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>07:26</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>76</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>07:27</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>44</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>52</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>52</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>06:10:41</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>07:36</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>86</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>07:37</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>54</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>07:55</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>72</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
           <t>07:59</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C53" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D46" t="n">
-        <v>109</v>
-      </c>
-      <c r="E46" t="inlineStr">
+      <c r="D53" t="n">
+        <v>76</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>08:11</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>88</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>94</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>99</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>105</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>115</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>118</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>118</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1506,7 +1856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1519,14 +1869,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:10:41</t>
+          <t>Última actualización: 06:43:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -1760,23 +2110,123 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>06:56</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>13</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>06:10:41</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>07:19</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>69</v>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>07:20</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>37</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>52</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>115</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1793,7 +2243,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1806,14 +2256,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:10:41</t>
+          <t>Última actualización: 06:43:00</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 2</t>
+          <t>Total filas: 4</t>
         </is>
       </c>
     </row>
@@ -1889,6 +2339,56 @@
         <v>93</v>
       </c>
       <c r="E7" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>07:44</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>61</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:33</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>110</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4588
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:00</t>
+          <t>Última actualización: 06:59:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 66</t>
         </is>
       </c>
     </row>
@@ -1323,7 +1323,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1348,21 +1348,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>07:19</t>
+          <t>07:18</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>69</v>
+        <v>19</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,21 +1398,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>07:20</t>
+          <t>07:19</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>70</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1448,12 +1448,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>07:21</t>
+          <t>07:20</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1462,7 +1462,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1473,21 +1473,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:21</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>76</v>
+        <v>38</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1498,12 +1498,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1512,7 +1512,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1528,16 +1528,16 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,21 +1573,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>86</v>
+        <v>35</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1603,16 +1603,16 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1628,16 +1628,16 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>72</v>
+        <v>52</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>76</v>
+        <v>37</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1678,16 +1678,16 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1728,16 +1728,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>105</v>
+        <v>60</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>115</v>
+        <v>61</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>118</v>
+        <v>72</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,23 +1823,298 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>08:17</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>78</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>08:21</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>82</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
           <t>06:43:00</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>08:22</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>99</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>08:27</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>88</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>08:28</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>105</v>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>98</v>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>08:38</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>115</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>08:40</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>101</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>08:41</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>102</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D60" t="n">
+      <c r="D69" t="n">
         <v>118</v>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>115</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>117</v>
+      </c>
+      <c r="E71" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1856,7 +2131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1869,14 +2144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:00</t>
+          <t>Última actualización: 06:59:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2410,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -2149,7 +2424,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>69</v>
+        <v>20</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -2185,12 +2460,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2199,7 +2474,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2215,18 +2490,118 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
+          <t>07:35</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>52</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>08:37</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>98</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>06:43:00</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>08:38</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D20" t="n">
         <v>115</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>115</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>117</v>
+      </c>
+      <c r="E22" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2243,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2256,14 +2631,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:43:00</t>
+          <t>Última actualización: 06:59:54</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 6</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2697,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:10:41</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2336,7 +2711,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>93</v>
+        <v>44</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2372,25 +2747,75 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>08:32</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>93</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>06:43:00</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>08:33</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>110</v>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>06:59:54</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>08:47</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>108</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4589
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E71"/>
+  <dimension ref="A1:E76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:54</t>
+          <t>Última actualización: 07:22:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 66</t>
+          <t>Total filas: 71</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1498,21 +1498,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>07:26</t>
+          <t>07:22</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>27</v>
+        <v>0</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1523,12 +1523,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>07:27</t>
+          <t>07:26</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1537,7 +1537,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>44</v>
+        <v>4</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1548,21 +1548,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>07:34</t>
+          <t>07:27</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1573,7 +1573,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1583,11 +1583,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1598,21 +1598,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>07:35</t>
+          <t>07:34</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>52</v>
+        <v>12</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1648,21 +1648,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>07:36</t>
+          <t>07:35</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1673,12 +1673,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>07:37</t>
+          <t>07:36</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>54</v>
+        <v>14</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1698,21 +1698,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:37</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1723,12 +1723,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,21 +1748,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1803,16 +1803,16 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,21 +1823,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1848,21 +1848,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>82</v>
+        <v>49</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:27</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>88</v>
+        <v>59</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1928,16 +1928,16 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -1998,21 +1998,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,12 +2048,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>118</v>
+        <v>78</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2098,23 +2098,148 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>08:41</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>79</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>07:22:52</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>08:54</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>92</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>07:22:52</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
           <t>08:56</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D71" t="n">
-        <v>117</v>
-      </c>
-      <c r="E71" t="inlineStr">
+      <c r="D73" t="n">
+        <v>94</v>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>07:22:52</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>104</v>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>07:22:52</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>114</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>07:22:52</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:17</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>115</v>
+      </c>
+      <c r="E76" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2144,7 +2269,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:54</t>
+          <t>Última actualización: 07:22:52</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2585,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2474,7 +2599,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -2510,7 +2635,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2524,7 +2649,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>98</v>
+        <v>75</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2560,7 +2685,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2574,7 +2699,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>115</v>
+        <v>92</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2585,7 +2710,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2599,7 +2724,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>117</v>
+        <v>94</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2631,7 +2756,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 06:59:54</t>
+          <t>Última actualización: 07:22:52</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2822,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2711,7 +2836,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -2747,7 +2872,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2761,7 +2886,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>93</v>
+        <v>70</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -2797,7 +2922,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2811,7 +2936,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4590
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E76"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:52</t>
+          <t>Última actualización: 07:45:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 71</t>
+          <t>Total filas: 79</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1723,21 +1723,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>07:54</t>
+          <t>07:46</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>32</v>
+        <v>1</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1748,12 +1748,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>07:55</t>
+          <t>07:54</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1773,21 +1773,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>07:59</t>
+          <t>07:55</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1798,21 +1798,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>08:00</t>
+          <t>07:59</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>61</v>
+        <v>14</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1823,12 +1823,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>08:03</t>
+          <t>08:00</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1837,7 +1837,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>41</v>
+        <v>61</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -1853,16 +1853,16 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>08:11</t>
+          <t>08:03</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1873,21 +1873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>08:17</t>
+          <t>08:05</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>55</v>
+        <v>20</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -1898,21 +1898,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>08:21</t>
+          <t>08:11</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>59</v>
+        <v>26</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,21 +1923,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>08:22</t>
+          <t>08:17</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>99</v>
+        <v>32</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,21 +1948,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>08:27</t>
+          <t>08:21</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -1978,16 +1978,16 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>08:28</t>
+          <t>08:22</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -2003,16 +2003,16 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>08:37</t>
+          <t>08:27</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2023,21 +2023,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>08:38</t>
+          <t>08:28</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>115</v>
+        <v>43</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2053,16 +2053,16 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:37</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2073,21 +2073,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:38</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>118</v>
+        <v>53</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2103,16 +2103,16 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,21 +2123,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,21 +2148,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>94</v>
+        <v>56</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>114</v>
+        <v>71</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,23 +2223,223 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>09:06</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>81</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>09:11</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>86</v>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
           <t>07:22:52</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>114</v>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
         <is>
           <t>09:17</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D76" t="n">
-        <v>115</v>
-      </c>
-      <c r="E76" t="inlineStr">
+      <c r="D79" t="n">
+        <v>92</v>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>101</v>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>09:26</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>101</v>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>113</v>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>116</v>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>118</v>
+      </c>
+      <c r="E84" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2269,7 +2469,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:52</t>
+          <t>Última actualización: 07:45:26</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2860,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2674,7 +2874,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>115</v>
+        <v>53</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2685,7 +2885,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2699,7 +2899,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2710,7 +2910,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2724,7 +2924,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>94</v>
+        <v>71</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -2743,7 +2943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2756,14 +2956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:22:52</t>
+          <t>Última actualización: 07:45:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 6</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -2897,7 +3097,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2911,7 +3111,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>110</v>
+        <v>48</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -2941,6 +3141,56 @@
       <c r="E11" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>08:48</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>63</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>07:45:25</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:28</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>103</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4591
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:26</t>
+          <t>Última actualización: 07:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 79</t>
+          <t>Total filas: 82</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -1798,7 +1798,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1812,7 +1812,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -1862,7 +1862,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -1898,7 +1898,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -1912,7 +1912,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -1923,7 +1923,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2048,7 +2048,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2187,7 +2187,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2212,7 +2212,7 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2262,7 +2262,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>86</v>
+        <v>72</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2298,7 +2298,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,7 +2348,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2358,11 +2358,11 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>116</v>
+        <v>99</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,23 +2423,98 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>102</v>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
           <t>09:43</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D84" t="n">
+      <c r="D85" t="n">
+        <v>104</v>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>117</v>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
         <v>118</v>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E87" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2456,7 +2531,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2469,14 +2544,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:26</t>
+          <t>Última actualización: 07:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2910,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2849,7 +2924,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>75</v>
+        <v>38</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -2885,7 +2960,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2899,7 +2974,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>69</v>
+        <v>55</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -2910,7 +2985,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2924,9 +2999,34 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>118</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2943,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2956,14 +3056,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:45:26</t>
+          <t>Última actualización: 07:59:51</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 8</t>
+          <t>Total filas: 9</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3172,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3086,7 +3186,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>70</v>
+        <v>33</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -3122,7 +3222,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3136,7 +3236,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>85</v>
+        <v>48</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -3172,23 +3272,48 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>09:27</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>88</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>07:45:25</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>09:28</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>103</v>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4592
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E87"/>
+  <dimension ref="A1:E96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:59:51</t>
+          <t>Última actualización: 08:20:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 82</t>
+          <t>Total filas: 91</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1948,7 +1948,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1962,7 +1962,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2023,7 +2023,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2037,7 +2037,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -2073,7 +2073,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2123,7 +2123,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2133,11 +2133,11 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,7 +2148,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2158,11 +2158,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2228,16 +2228,16 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2248,21 +2248,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>114</v>
+        <v>46</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,21 +2298,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,12 +2323,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2337,7 +2337,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>79</v>
+        <v>114</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>87</v>
+        <v>57</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,12 +2373,12 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -2387,7 +2387,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2403,16 +2403,16 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2428,16 +2428,16 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>117</v>
+        <v>67</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,23 +2498,248 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>09:38</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>78</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
           <t>07:59:51</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>09:41</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>102</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>82</v>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>09:43</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>83</v>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>09:56</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>96</v>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
         <is>
           <t>09:57</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D87" t="n">
+      <c r="D92" t="n">
         <v>118</v>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>98</v>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>100</v>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>112</v>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>113</v>
+      </c>
+      <c r="E96" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2531,7 +2756,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2544,14 +2769,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:59:51</t>
+          <t>Última actualización: 08:20:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3160,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2949,7 +3174,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2985,21 +3210,21 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3015,18 +3240,93 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>08:56</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>57</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>08:57</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>37</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>09:57</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D23" t="n">
+      <c r="D25" t="n">
         <v>118</v>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>98</v>
+      </c>
+      <c r="E26" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3043,7 +3343,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3056,14 +3356,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:59:51</t>
+          <t>Última actualización: 08:20:07</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 9</t>
+          <t>Total filas: 10</t>
         </is>
       </c>
     </row>
@@ -3197,7 +3497,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3211,7 +3511,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -3247,7 +3547,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3261,7 +3561,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>28</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -3297,7 +3597,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3311,11 +3611,36 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>103</v>
+        <v>68</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>08:20:07</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10:08</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>108</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4593
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E96"/>
+  <dimension ref="A1:E103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:20:07</t>
+          <t>Última actualización: 08:39:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 91</t>
+          <t>Total filas: 98</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2098,21 +2098,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>08:40</t>
+          <t>08:39</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>78</v>
+        <v>0</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2123,12 +2123,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:39</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2148,12 +2148,12 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:22:52</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>08:41</t>
+          <t>08:40</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -2162,7 +2162,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>21</v>
+        <v>78</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2173,21 +2173,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,21 +2198,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>08:41</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>35</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,21 +2223,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>57</v>
+        <v>15</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2253,16 +2253,16 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,21 +2273,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>46</v>
+        <v>17</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2303,16 +2303,16 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>07:22:52</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>114</v>
+        <v>26</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2348,21 +2348,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2378,16 +2378,16 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,12 +2398,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2412,7 +2412,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>87</v>
+        <v>38</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,12 +2448,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,21 +2473,21 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>102</v>
+        <v>47</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2553,16 +2553,16 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:42</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>83</v>
+        <v>52</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>96</v>
+        <v>59</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>118</v>
+        <v>62</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2653,16 +2653,16 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>98</v>
+        <v>82</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>10:12</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,23 +2723,198 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
+          <t>07:59:51</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>118</v>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>09:58</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>79</v>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
           <t>08:20:07</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>100</v>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>82</v>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>93</v>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
         <is>
           <t>10:13</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D96" t="n">
-        <v>113</v>
-      </c>
-      <c r="E96" t="inlineStr">
+      <c r="D101" t="n">
+        <v>94</v>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>107</v>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>108</v>
+      </c>
+      <c r="E103" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2756,7 +2931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2769,14 +2944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:20:07</t>
+          <t>Última actualización: 08:39:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 22</t>
         </is>
       </c>
     </row>
@@ -3185,21 +3360,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>08:54</t>
+          <t>08:39</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -3210,12 +3385,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>08:55</t>
+          <t>08:54</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3224,7 +3399,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3235,21 +3410,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>57</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -3260,12 +3435,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3274,7 +3449,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3285,21 +3460,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>118</v>
+        <v>37</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3310,23 +3485,48 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>118</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>98</v>
-      </c>
-      <c r="E26" t="inlineStr">
+      <c r="D27" t="n">
+        <v>79</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3343,7 +3543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3356,14 +3556,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:20:07</t>
+          <t>Última actualización: 08:39:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 10</t>
+          <t>Total filas: 12</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3747,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3561,7 +3761,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -3597,7 +3797,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3611,7 +3811,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3622,7 +3822,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3636,11 +3836,61 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>109</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>10:35</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>116</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4594
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:39:26</t>
+          <t>Última actualización: 08:54:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 98</t>
+          <t>Total filas: 104</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2223,7 +2223,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2237,7 +2237,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -2273,12 +2273,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2287,7 +2287,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2298,12 +2298,12 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -2312,7 +2312,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2323,21 +2323,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>09:05</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2353,16 +2353,16 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>09:06</t>
+          <t>09:05</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -2373,21 +2373,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>09:11</t>
+          <t>09:06</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>51</v>
+        <v>12</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2398,21 +2398,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>09:16</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,21 +2423,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:11</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2448,21 +2448,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:12</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2473,12 +2473,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,12 +2498,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -2512,7 +2512,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>101</v>
+        <v>23</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2523,21 +2523,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2548,21 +2548,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,21 +2573,21 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>52</v>
+        <v>101</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,21 +2598,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:42</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>82</v>
+        <v>37</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>64</v>
+        <v>44</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2698,21 +2698,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>77</v>
+        <v>47</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>79</v>
+        <v>49</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>100</v>
+        <v>62</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>118</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2823,21 +2823,21 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>10:12</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,21 +2848,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>107</v>
+        <v>67</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2898,23 +2898,173 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>10:11</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>77</v>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>08:39:26</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>93</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>79</v>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>92</v>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
         <is>
           <t>10:27</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D103" t="n">
-        <v>108</v>
-      </c>
-      <c r="E103" t="inlineStr">
+      <c r="D107" t="n">
+        <v>93</v>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D108" t="n">
+        <v>109</v>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10:44</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>110</v>
+      </c>
+      <c r="E109" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -2931,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2944,14 +3094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:39:26</t>
+          <t>Última actualización: 08:54:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 22</t>
+          <t>Total filas: 23</t>
         </is>
       </c>
     </row>
@@ -3385,7 +3535,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3399,7 +3549,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -3435,12 +3585,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>08:56</t>
+          <t>08:55</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3449,7 +3599,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3460,12 +3610,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>08:57</t>
+          <t>08:56</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3474,7 +3624,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3485,21 +3635,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>08:57</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>118</v>
+        <v>37</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -3510,23 +3660,48 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>09:57</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>118</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>09:58</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>79</v>
-      </c>
-      <c r="E27" t="inlineStr">
+      <c r="D28" t="n">
+        <v>64</v>
+      </c>
+      <c r="E28" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3543,7 +3718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3556,14 +3731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:39:26</t>
+          <t>Última actualización: 08:54:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 12</t>
+          <t>Total filas: 13</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3972,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3811,7 +3986,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -3847,48 +4022,73 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:28</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>94</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>116</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D18" t="n">
+        <v>101</v>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4595
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E109"/>
+  <dimension ref="A1:E123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:54:24</t>
+          <t>Última actualización: 09:14:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 104</t>
+          <t>Total filas: 118</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2473,7 +2473,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2487,7 +2487,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>37</v>
+        <v>2</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2498,21 +2498,21 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>09:17</t>
+          <t>09:16</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2548,12 +2548,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>09:18</t>
+          <t>09:17</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2562,7 +2562,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2573,12 +2573,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>07:59:51</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>09:26</t>
+          <t>09:18</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -2587,7 +2587,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>101</v>
+        <v>79</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2612,7 +2612,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>32</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,21 +2623,21 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>09:27</t>
+          <t>09:26</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2648,21 +2648,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>09:31</t>
+          <t>09:27</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>37</v>
+        <v>67</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2673,21 +2673,21 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>09:38</t>
+          <t>09:31</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2703,16 +2703,16 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>09:41</t>
+          <t>09:38</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2723,21 +2723,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>09:42</t>
+          <t>09:40</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>82</v>
+        <v>26</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2748,21 +2748,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>09:43</t>
+          <t>09:41</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2773,21 +2773,21 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>09:56</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>62</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,21 +2798,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>09:57</t>
+          <t>09:42</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>118</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2828,16 +2828,16 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>09:58</t>
+          <t>09:43</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -2848,12 +2848,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -2862,7 +2862,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>100</v>
+        <v>41</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -2873,21 +2873,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>10:01</t>
+          <t>09:55</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>67</v>
+        <v>41</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -2903,16 +2903,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>10:11</t>
+          <t>09:56</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -2923,21 +2923,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>10:12</t>
+          <t>09:57</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>93</v>
+        <v>43</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -2953,16 +2953,16 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>10:13</t>
+          <t>09:58</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>79</v>
+        <v>64</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -2973,21 +2973,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -2998,21 +2998,21 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:01</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>93</v>
+        <v>47</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,21 +3023,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:11</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>109</v>
+        <v>57</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,23 +3048,373 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
+          <t>08:39:26</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D109" t="n">
+        <v>93</v>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>10:12</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D110" t="n">
+        <v>58</v>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
           <t>08:54:24</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D111" t="n">
+        <v>79</v>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D112" t="n">
+        <v>71</v>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D113" t="n">
+        <v>92</v>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>10:26</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D114" t="n">
+        <v>72</v>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D115" t="n">
+        <v>93</v>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>10:42</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D116" t="n">
+        <v>88</v>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D117" t="n">
+        <v>89</v>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>10:43</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>15_P INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="D118" t="n">
+        <v>109</v>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
         <is>
           <t>10:44</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D109" t="n">
+      <c r="D119" t="n">
         <v>110</v>
       </c>
-      <c r="E109" t="inlineStr">
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D120" t="n">
+        <v>102</v>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D121" t="n">
+        <v>103</v>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>104</v>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>11:09</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>115</v>
+      </c>
+      <c r="E123" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3094,7 +3444,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:54:24</t>
+          <t>Última actualización: 09:14:58</t>
         </is>
       </c>
     </row>
@@ -3660,7 +4010,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3674,7 +4024,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>118</v>
+        <v>43</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3718,7 +4068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3731,14 +4081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 08:54:24</t>
+          <t>Última actualización: 09:14:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 13</t>
+          <t>Total filas: 16</t>
         </is>
       </c>
     </row>
@@ -3947,7 +4297,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07:59:51</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3961,7 +4311,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>88</v>
+        <v>13</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -3997,12 +4347,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10:08</t>
+          <t>10:07</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -4011,7 +4361,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -4022,12 +4372,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>10:09</t>
+          <t>10:08</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -4036,7 +4386,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>75</v>
+        <v>89</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -4052,43 +4402,118 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10:28</t>
+          <t>10:09</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>215A_LA PLATA</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>94</v>
+        <v>75</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>73</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>08:54:24</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>10:28</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>94</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>10:34</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>80</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08:54:24</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
         <is>
           <t>10:35</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D18" t="n">
+      <c r="D21" t="n">
         <v>101</v>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4596
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E123"/>
+  <dimension ref="A1:E137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:58</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 118</t>
+          <t>Total filas: 132</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2998,7 +2998,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -3012,7 +3012,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -3023,7 +3023,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -3037,7 +3037,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>57</v>
+        <v>11</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3098,7 +3098,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -3112,7 +3112,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -3123,7 +3123,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -3133,11 +3133,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -3148,12 +3148,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>10:26</t>
+          <t>10:25</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -3162,7 +3162,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>92</v>
+        <v>25</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,12 +3198,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>10:27</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -3212,7 +3212,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,21 +3223,21 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>10:42</t>
+          <t>10:26</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3248,21 +3248,21 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:27</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>89</v>
+        <v>27</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -3273,12 +3273,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:42</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3287,7 +3287,7 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,12 +3298,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3312,7 +3312,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>110</v>
+        <v>43</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3323,21 +3323,21 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>102</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>104</v>
+        <v>55</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,23 +3398,373 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>10:56</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>56</v>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
           <t>09:14:58</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>10:57</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>103</v>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>58</v>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>10:58</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>104</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>11:02</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>62</v>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>09:14:58</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
         <is>
           <t>11:09</t>
         </is>
       </c>
-      <c r="C123" t="inlineStr">
+      <c r="C128" t="inlineStr">
         <is>
           <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
-      <c r="D123" t="n">
+      <c r="D128" t="n">
         <v>115</v>
       </c>
-      <c r="E123" t="inlineStr">
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>11:10</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>70</v>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>73</v>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>225_C ROCA-H SUR</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>73</v>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>11:19</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>79</v>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>87</v>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>98</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>102</v>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>112</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>118</v>
+      </c>
+      <c r="E137" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3431,7 +3781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3444,14 +3794,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:58</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 23</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -4052,6 +4402,56 @@
         <v>64</v>
       </c>
       <c r="E28" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>87</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>98</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4068,7 +4468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4081,14 +4481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 09:14:58</t>
+          <t>Última actualización: 10:00:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 16</t>
+          <t>Total filas: 17</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4747,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -4361,7 +4761,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>53</v>
+        <v>7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -4422,7 +4822,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -4436,7 +4836,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4472,7 +4872,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -4486,7 +4886,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -4516,6 +4916,31 @@
       <c r="E21" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>10:00:55</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>87</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4597
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E137"/>
+  <dimension ref="A1:E149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 132</t>
+          <t>Total filas: 144</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3273,21 +3273,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>10:42</t>
+          <t>10:38</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -3298,21 +3298,21 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>10:43</t>
+          <t>10:42</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -3333,7 +3333,7 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
@@ -3348,21 +3348,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>10:44</t>
+          <t>10:43</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>110</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3373,21 +3373,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>10:55</t>
+          <t>10:44</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -3398,21 +3398,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>10:56</t>
+          <t>10:51</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>56</v>
+        <v>13</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -3423,21 +3423,21 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>10:57</t>
+          <t>10:55</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>103</v>
+        <v>17</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -3448,21 +3448,21 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:56</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -3478,16 +3478,16 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>62</v>
+        <v>104</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,21 +3523,21 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>11:09</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>115</v>
+        <v>20</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3553,16 +3553,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>70</v>
+        <v>62</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,21 +3573,21 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>73</v>
+        <v>27</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:09</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>73</v>
+        <v>115</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>79</v>
+        <v>32</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3678,16 +3678,16 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>98</v>
+        <v>73</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>102</v>
+        <v>36</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>112</v>
+        <v>79</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,23 +3748,323 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>42</v>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>47</v>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>49</v>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>60</v>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>11:42</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D141" t="n">
+        <v>64</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>11:46</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D142" t="n">
+        <v>68</v>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
           <t>10:00:55</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>11:52</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D143" t="n">
+        <v>112</v>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>11:53</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D144" t="n">
+        <v>75</v>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
         <is>
           <t>11:58</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C145" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D137" t="n">
+      <c r="D145" t="n">
+        <v>80</v>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D146" t="n">
+        <v>90</v>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D147" t="n">
+        <v>97</v>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>109</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
         <v>118</v>
       </c>
-      <c r="E137" t="inlineStr">
+      <c r="E149" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -3781,7 +4081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3794,14 +4094,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:41</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4710,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -4424,7 +4724,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -4435,7 +4735,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4449,9 +4749,34 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>98</v>
+        <v>60</v>
       </c>
       <c r="E30" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>109</v>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4481,7 +4806,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:00:55</t>
+          <t>Última actualización: 10:38:41</t>
         </is>
       </c>
     </row>
@@ -4922,7 +5247,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -4936,7 +5261,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>87</v>
+        <v>49</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4598
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E149"/>
+  <dimension ref="A1:E161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:41</t>
+          <t>Última actualización: 10:55:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 144</t>
+          <t>Total filas: 156</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3498,21 +3498,21 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>10:58</t>
+          <t>10:57</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>104</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>20</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,21 +3548,21 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>11:02</t>
+          <t>10:58</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>62</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3573,12 +3573,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>11:05</t>
+          <t>11:02</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3587,7 +3587,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>27</v>
+        <v>62</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -3598,21 +3598,21 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>11:09</t>
+          <t>11:05</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>115</v>
+        <v>27</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -3623,21 +3623,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>11:10</t>
+          <t>11:08</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -3648,21 +3648,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:09</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>35</v>
+        <v>115</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3673,21 +3673,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:10</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D134" t="n">
-        <v>73</v>
+        <v>15</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -3698,21 +3698,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3728,16 +3728,16 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,21 +3748,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>47</v>
+        <v>79</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,21 +3798,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>49</v>
+        <v>25</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3823,21 +3823,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>60</v>
+        <v>30</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3853,16 +3853,16 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,21 +3873,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D142" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>112</v>
+        <v>43</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>75</v>
+        <v>46</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>80</v>
+        <v>47</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3978,16 +3978,16 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>90</v>
+        <v>68</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>97</v>
+        <v>112</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,23 +4048,323 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>60</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>11:58</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>63</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>73</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
           <t>10:38:41</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>97</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>12:22</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>87</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>12:23</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D154" t="n">
+        <v>88</v>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D155" t="n">
+        <v>109</v>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D156" t="n">
+        <v>93</v>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D157" t="n">
+        <v>96</v>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>10:38:41</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
         <is>
           <t>12:36</t>
         </is>
       </c>
-      <c r="C149" t="inlineStr">
+      <c r="C158" t="inlineStr">
         <is>
           <t>27_EL RETIRO</t>
         </is>
       </c>
-      <c r="D149" t="n">
+      <c r="D158" t="n">
         <v>118</v>
       </c>
-      <c r="E149" t="inlineStr">
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D159" t="n">
+        <v>102</v>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D160" t="n">
+        <v>103</v>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>107</v>
+      </c>
+      <c r="E161" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4081,7 +4381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4094,14 +4394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:41</t>
+          <t>Última actualización: 10:55:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 28</t>
         </is>
       </c>
     </row>
@@ -4560,7 +4860,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4570,11 +4870,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4585,7 +4885,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4595,11 +4895,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -4735,21 +5035,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -4760,23 +5060,73 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>11:38</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>43</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>10:38:41</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>12:27</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D32" t="n">
         <v>109</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:28</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>93</v>
+      </c>
+      <c r="E33" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4793,7 +5143,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4806,14 +5156,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:38:41</t>
+          <t>Última actualización: 10:55:24</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 17</t>
+          <t>Total filas: 18</t>
         </is>
       </c>
     </row>
@@ -5264,6 +5614,31 @@
         <v>49</v>
       </c>
       <c r="E22" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11:28</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>33</v>
+      </c>
+      <c r="E23" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4599
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E161"/>
+  <dimension ref="A1:E167"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:55:24</t>
+          <t>Última actualización: 11:09:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 156</t>
+          <t>Total filas: 162</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -3662,7 +3662,7 @@
         </is>
       </c>
       <c r="D133" t="n">
-        <v>115</v>
+        <v>0</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -3698,12 +3698,12 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>11:13</t>
+          <t>11:12</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -3712,7 +3712,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>18</v>
+        <v>3</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>73</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,12 +3748,12 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>11:14</t>
+          <t>11:13</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -3762,7 +3762,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>19</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3773,21 +3773,21 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>11:19</t>
+          <t>11:14</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>79</v>
+        <v>19</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -3798,12 +3798,12 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>11:20</t>
+          <t>11:19</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -3812,7 +3812,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -3828,16 +3828,16 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>11:25</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -3848,21 +3848,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>11:27</t>
+          <t>11:25</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -3873,12 +3873,12 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>11:28</t>
+          <t>11:27</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -3903,16 +3903,16 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:28</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -3923,21 +3923,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3948,21 +3948,21 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>47</v>
+        <v>32</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>68</v>
+        <v>33</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>112</v>
+        <v>68</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,12 +4023,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -4037,7 +4037,7 @@
         </is>
       </c>
       <c r="D148" t="n">
-        <v>58</v>
+        <v>43</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4053,16 +4053,16 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,21 +4123,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>87</v>
+        <v>59</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>109</v>
+        <v>72</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>93</v>
+        <v>73</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4253,16 +4253,16 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D157" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,21 +4273,21 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>102</v>
+        <v>78</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4328,16 +4328,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>103</v>
+        <v>93</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4353,18 +4353,168 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D161" t="n">
+        <v>96</v>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>12:32</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D162" t="n">
+        <v>83</v>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>12:36</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D163" t="n">
+        <v>87</v>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>10:55:24</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D164" t="n">
+        <v>102</v>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D165" t="n">
+        <v>89</v>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
           <t>12:42</t>
         </is>
       </c>
-      <c r="C161" t="inlineStr">
+      <c r="C166" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D161" t="n">
+      <c r="D166" t="n">
+        <v>93</v>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
         <v>107</v>
       </c>
-      <c r="E161" t="inlineStr">
+      <c r="E167" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4394,7 +4544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:55:24</t>
+          <t>Última actualización: 11:09:58</t>
         </is>
       </c>
     </row>
@@ -4860,7 +5010,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -4870,11 +5020,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -4885,7 +5035,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -4895,11 +5045,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5010,7 +5160,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -5024,7 +5174,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -5060,7 +5210,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -5074,7 +5224,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5085,7 +5235,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -5099,7 +5249,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5143,7 +5293,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5156,14 +5306,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 10:55:24</t>
+          <t>Última actualización: 11:09:58</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 18</t>
+          <t>Total filas: 19</t>
         </is>
       </c>
     </row>
@@ -5597,7 +5747,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -5611,7 +5761,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -5639,6 +5789,31 @@
         <v>33</v>
       </c>
       <c r="E23" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>11:09:57</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>108</v>
+      </c>
+      <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4600
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E167"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:58</t>
+          <t>Última actualización: 11:34:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 162</t>
+          <t>Total filas: 170</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -3923,12 +3923,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -3937,7 +3937,7 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -3953,16 +3953,16 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>11:41</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -3973,21 +3973,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>11:42</t>
+          <t>11:41</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -3998,21 +3998,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>11:46</t>
+          <t>11:42</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>68</v>
+        <v>8</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -4023,21 +4023,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>11:52</t>
+          <t>11:46</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>43</v>
+        <v>68</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -4048,12 +4048,12 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>11:53</t>
+          <t>11:52</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -4062,7 +4062,7 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -4073,21 +4073,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>11:55</t>
+          <t>11:53</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,21 +4098,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>11:57</t>
+          <t>11:55</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>48</v>
+        <v>21</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4123,12 +4123,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>11:58</t>
+          <t>11:57</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -4137,7 +4137,7 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>63</v>
+        <v>48</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -4148,21 +4148,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>12:08</t>
+          <t>11:58</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D153" t="n">
-        <v>59</v>
+        <v>24</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,21 +4173,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:08</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>97</v>
+        <v>34</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,21 +4198,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>12:21</t>
+          <t>12:10</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>72</v>
+        <v>36</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4223,21 +4223,21 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -4248,12 +4248,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>12:22</t>
+          <t>12:21</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>87</v>
+        <v>72</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -4273,12 +4273,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>12:23</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>88</v>
+        <v>48</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,21 +4298,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>12:22</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4328,16 +4328,16 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>12:28</t>
+          <t>12:23</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -4348,21 +4348,21 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:25</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -4373,21 +4373,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:27</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>83</v>
+        <v>53</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4398,21 +4398,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:28</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -4428,16 +4428,16 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,21 +4448,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>89</v>
+        <v>58</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,21 +4473,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>93</v>
+        <v>62</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,23 +4498,223 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
+          <t>12:37</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>102</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>12:38</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D168" t="n">
+        <v>64</v>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>68</v>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>12:56</t>
         </is>
       </c>
-      <c r="C167" t="inlineStr">
+      <c r="C170" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D167" t="n">
-        <v>107</v>
-      </c>
-      <c r="E167" t="inlineStr">
+      <c r="D170" t="n">
+        <v>82</v>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>83</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>99</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>99</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>110</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>118</v>
+      </c>
+      <c r="E175" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4531,7 +4731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4544,14 +4744,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:58</t>
+          <t>Última actualización: 11:34:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 28</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -5210,12 +5410,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>11:38</t>
+          <t>11:37</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -5224,7 +5424,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>29</v>
+        <v>3</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5240,16 +5440,16 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>12:27</t>
+          <t>11:38</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5260,23 +5460,98 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12:27</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>53</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>10:55:24</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>12:28</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D33" t="n">
+      <c r="D34" t="n">
         <v>93</v>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12:57</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>83</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>110</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5293,7 +5568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5306,14 +5581,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:09:58</t>
+          <t>Última actualización: 11:34:57</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 19</t>
+          <t>Total filas: 20</t>
         </is>
       </c>
     </row>
@@ -5797,7 +6072,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5811,11 +6086,36 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>108</v>
+        <v>83</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>11:34:57</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>114</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4601
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E175"/>
+  <dimension ref="A1:E180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:34:57</t>
+          <t>Última actualización: 11:52:55</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 170</t>
+          <t>Total filas: 175</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4073,7 +4073,7 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -4087,7 +4087,7 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>58</v>
+        <v>1</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -4098,7 +4098,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -4112,7 +4112,7 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>21</v>
+        <v>3</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -4148,7 +4148,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -4162,7 +4162,7 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>48</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>30</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4423,21 +4423,21 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>12:31</t>
+          <t>12:29</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>96</v>
+        <v>37</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -4448,12 +4448,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -4462,7 +4462,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>58</v>
+        <v>39</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4478,16 +4478,16 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,12 +4498,12 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -4512,7 +4512,7 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>102</v>
+        <v>44</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>82</v>
+        <v>50</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>99</v>
+        <v>65</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>99</v>
+        <v>81</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>110</v>
+        <v>81</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,23 +4698,148 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>13:23</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>91</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>11:52:55</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>13:24</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>92</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>11:52:55</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
           <t>13:32</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
+      <c r="C177" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D175" t="n">
-        <v>118</v>
-      </c>
-      <c r="E175" t="inlineStr">
+      <c r="D177" t="n">
+        <v>100</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>11:52:55</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>108</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>11:52:55</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>115</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>11:52:55</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>13:49</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>117</v>
+      </c>
+      <c r="E180" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4744,7 +4869,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:34:57</t>
+          <t>Última actualización: 11:52:55</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5585,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5474,7 +5599,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>53</v>
+        <v>35</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5510,7 +5635,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5524,7 +5649,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -5535,7 +5660,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5549,7 +5674,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>110</v>
+        <v>92</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5581,7 +5706,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:34:57</t>
+          <t>Última actualización: 11:52:55</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6197,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6086,7 +6211,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>83</v>
+        <v>65</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6097,7 +6222,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6111,7 +6236,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>114</v>
+        <v>96</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4602
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E180"/>
+  <dimension ref="A1:E183"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:52:55</t>
+          <t>Última actualización: 12:08:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 175</t>
+          <t>Total filas: 178</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -4187,7 +4187,7 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -4198,7 +4198,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -4212,7 +4212,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>30</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4373,7 +4373,7 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -4387,7 +4387,7 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -4448,7 +4448,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -4458,11 +4458,11 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -4473,12 +4473,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>11:34:57</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>12:32</t>
+          <t>12:31</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -4487,7 +4487,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -4498,21 +4498,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>11:34:57</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:32</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>44</v>
+        <v>58</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -4523,12 +4523,12 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -4537,7 +4537,7 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,21 +4548,21 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>46</v>
+        <v>102</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>64</v>
+        <v>34</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>81</v>
+        <v>48</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>81</v>
+        <v>49</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,21 +4698,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4753,16 +4753,16 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>108</v>
+        <v>76</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>115</v>
+        <v>80</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,23 +4823,98 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>84</v>
+      </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>12:08:56</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>92</v>
+      </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>12:08:56</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>99</v>
+      </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>12:08:56</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
           <t>13:49</t>
         </is>
       </c>
-      <c r="C180" t="inlineStr">
+      <c r="C183" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D180" t="n">
-        <v>117</v>
-      </c>
-      <c r="E180" t="inlineStr">
+      <c r="D183" t="n">
+        <v>101</v>
+      </c>
+      <c r="E183" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4869,7 +4944,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:52:55</t>
+          <t>Última actualización: 12:08:56</t>
         </is>
       </c>
     </row>
@@ -5585,7 +5660,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -5599,7 +5674,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5635,7 +5710,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5649,7 +5724,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -5660,7 +5735,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -5674,7 +5749,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -5693,7 +5768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5706,14 +5781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 11:52:55</t>
+          <t>Última actualización: 12:08:56</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 20</t>
+          <t>Total filas: 21</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6272,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6211,7 +6286,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6222,7 +6297,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -6236,11 +6311,36 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>96</v>
+        <v>80</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>12:08:56</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>13:52</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>104</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4603
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E183"/>
+  <dimension ref="A1:E193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:56</t>
+          <t>Última actualización: 12:32:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 178</t>
+          <t>Total filas: 188</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4523,21 +4523,21 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>12:36</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
@@ -4548,12 +4548,12 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>12:37</t>
+          <t>12:36</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -4562,7 +4562,7 @@
         </is>
       </c>
       <c r="D169" t="n">
-        <v>102</v>
+        <v>28</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -4573,21 +4573,21 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>12:38</t>
+          <t>12:37</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -4598,21 +4598,21 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>12:42</t>
+          <t>12:38</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
@@ -4623,21 +4623,21 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>12:55</t>
+          <t>12:42</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>47</v>
+        <v>10</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
@@ -4648,21 +4648,21 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>12:56</t>
+          <t>12:55</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D173" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,21 +4673,21 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>12:57</t>
+          <t>12:56</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>49</v>
+        <v>24</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4703,16 +4703,16 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:57</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D175" t="n">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4723,21 +4723,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>65</v>
+        <v>26</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -4748,21 +4748,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D177" t="n">
-        <v>91</v>
+        <v>65</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,21 +4773,21 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>76</v>
+        <v>41</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>80</v>
+        <v>42</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,21 +4823,21 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>99</v>
+        <v>53</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,23 +4898,273 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>56</v>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>13:32</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>60</v>
+      </c>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>13:40</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>68</v>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>13:47</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>75</v>
+      </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
           <t>12:08:56</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B187" t="inlineStr">
         <is>
           <t>13:49</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
+      <c r="C187" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D183" t="n">
+      <c r="D187" t="n">
         <v>101</v>
       </c>
-      <c r="E183" t="inlineStr">
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>13:50</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>78</v>
+      </c>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>96</v>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>14:08</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D190" t="n">
+        <v>96</v>
+      </c>
+      <c r="E190" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D191" t="n">
+        <v>105</v>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>114</v>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>116</v>
+      </c>
+      <c r="E193" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -4931,7 +5181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4944,14 +5194,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:56</t>
+          <t>Última actualización: 12:32:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 33</t>
         </is>
       </c>
     </row>
@@ -5735,23 +5985,73 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>12:58</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>26</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>13:24</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>215A_EL PATO</t>
         </is>
       </c>
-      <c r="D36" t="n">
-        <v>76</v>
-      </c>
-      <c r="E36" t="inlineStr">
+      <c r="D37" t="n">
+        <v>52</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>116</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5768,7 +6068,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5781,14 +6081,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:08:56</t>
+          <t>Última actualización: 12:32:19</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 21</t>
+          <t>Total filas: 24</t>
         </is>
       </c>
     </row>
@@ -6297,25 +6597,25 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>12:58</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>215B_LP-P MOR-1 Y 57</t>
+          <t>215C_LA PLATA</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>80</v>
+        <v>26</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>L6173</t>
+          <t>L6203</t>
         </is>
       </c>
     </row>
@@ -6327,18 +6627,93 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>13:28</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>80</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>13:29</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>57</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>12:08:56</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>13:52</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D26" t="n">
+      <c r="D28" t="n">
         <v>104</v>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>116</v>
+      </c>
+      <c r="E29" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4604
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E193"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:32:19</t>
+          <t>Última actualización: 12:50:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 188</t>
+          <t>Total filas: 195</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4648,7 +4648,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D173" t="n">
-        <v>23</v>
+        <v>5</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
@@ -4673,7 +4673,7 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4687,7 +4687,7 @@
         </is>
       </c>
       <c r="D174" t="n">
-        <v>24</v>
+        <v>6</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -4698,7 +4698,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -4712,7 +4712,7 @@
         </is>
       </c>
       <c r="D175" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4787,7 +4787,7 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4812,7 +4812,7 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>42</v>
+        <v>24</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4823,12 +4823,12 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -4837,7 +4837,7 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>91</v>
+        <v>31</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,21 +4848,21 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>52</v>
+        <v>91</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4903,16 +4903,16 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,16 +4928,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>68</v>
+        <v>42</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>101</v>
+        <v>57</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,12 +5023,12 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>78</v>
+        <v>101</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,21 +5048,21 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>96</v>
+        <v>60</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>96</v>
+        <v>65</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,21 +5123,21 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>114</v>
+        <v>78</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,23 +5148,198 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D193" t="n">
+        <v>81</v>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>14:16</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D194" t="n">
+        <v>86</v>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
           <t>12:32:19</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>14:17</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D195" t="n">
+        <v>105</v>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>14:26</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D196" t="n">
+        <v>96</v>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D197" t="n">
+        <v>97</v>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>12:32:19</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr">
+      <c r="C198" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D193" t="n">
+      <c r="D198" t="n">
         <v>116</v>
       </c>
-      <c r="E193" t="inlineStr">
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>111</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>117</v>
+      </c>
+      <c r="E200" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5181,7 +5356,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E38"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5194,14 +5369,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:32:19</t>
+          <t>Última actualización: 12:50:45</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 33</t>
+          <t>Total filas: 35</t>
         </is>
       </c>
     </row>
@@ -5660,7 +5835,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5670,11 +5845,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5685,7 +5860,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5695,11 +5870,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5960,7 +6135,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -5974,7 +6149,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -6010,7 +6185,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6024,7 +6199,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>52</v>
+        <v>34</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6035,23 +6210,73 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>97</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>12:32:19</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D38" t="n">
+      <c r="D39" t="n">
         <v>116</v>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>12:50:45</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>14:47</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>117</v>
+      </c>
+      <c r="E40" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6081,7 +6306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:32:19</t>
+          <t>Última actualización: 12:50:45</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6797,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6586,7 +6811,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6622,7 +6847,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -6636,7 +6861,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>80</v>
+        <v>38</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -6672,7 +6897,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -6686,7 +6911,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>104</v>
+        <v>62</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4605
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E200"/>
+  <dimension ref="A1:E206"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:50:45</t>
+          <t>Última actualización: 13:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 195</t>
+          <t>Total filas: 201</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4748,12 +4748,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>13:13</t>
+          <t>13:11</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4762,7 +4762,7 @@
         </is>
       </c>
       <c r="D177" t="n">
-        <v>65</v>
+        <v>2</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>23</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,21 +4798,21 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>13:14</t>
+          <t>13:13</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4828,16 +4828,16 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>13:21</t>
+          <t>13:14</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
@@ -4848,12 +4848,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>11:52:55</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>13:23</t>
+          <t>13:21</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4862,7 +4862,7 @@
         </is>
       </c>
       <c r="D181" t="n">
-        <v>91</v>
+        <v>12</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
@@ -4873,21 +4873,21 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>11:52:55</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>13:24</t>
+          <t>13:23</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D182" t="n">
-        <v>34</v>
+        <v>91</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -4898,21 +4898,21 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>13:25</t>
+          <t>13:24</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D183" t="n">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -4928,16 +4928,16 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>13:28</t>
+          <t>13:25</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -4948,21 +4948,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>12:32:19</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>13:32</t>
+          <t>13:28</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -4973,21 +4973,21 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>13:40</t>
+          <t>13:32</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -4998,21 +4998,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>13:47</t>
+          <t>13:40</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,21 +5023,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>13:49</t>
+          <t>13:47</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>101</v>
+        <v>38</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5048,12 +5048,12 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>13:49</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -5062,7 +5062,7 @@
         </is>
       </c>
       <c r="D189" t="n">
-        <v>60</v>
+        <v>101</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -5073,21 +5073,21 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>13:55</t>
+          <t>13:50</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>65</v>
+        <v>41</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5098,21 +5098,21 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>14:08</t>
+          <t>13:55</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>78</v>
+        <v>46</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,21 +5148,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:08</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>81</v>
+        <v>59</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5178,16 +5178,16 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,12 +5198,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>12:50:45</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>105</v>
+        <v>86</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>116</v>
+        <v>77</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5303,16 +5303,16 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,23 +5323,173 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D200" t="n">
+        <v>79</v>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>14:41</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D201" t="n">
+        <v>92</v>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
           <t>12:50:45</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
+      <c r="B202" t="inlineStr">
         <is>
           <t>14:47</t>
         </is>
       </c>
-      <c r="C200" t="inlineStr">
+      <c r="C202" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D200" t="n">
+      <c r="D202" t="n">
         <v>117</v>
       </c>
-      <c r="E200" t="inlineStr">
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D203" t="n">
+        <v>99</v>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D204" t="n">
+        <v>108</v>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D205" t="n">
+        <v>112</v>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>15:07</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>118</v>
+      </c>
+      <c r="E206" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5356,7 +5506,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5369,14 +5519,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:50:45</t>
+          <t>Última actualización: 13:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 35</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -5835,7 +5985,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -5845,11 +5995,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5860,7 +6010,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -5870,11 +6020,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6185,7 +6335,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -6199,7 +6349,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -6235,7 +6385,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6249,7 +6399,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>116</v>
+        <v>79</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6277,6 +6427,56 @@
         <v>117</v>
       </c>
       <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>99</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>108</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6293,7 +6493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6306,14 +6506,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 12:50:45</t>
+          <t>Última actualización: 13:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 24</t>
+          <t>Total filas: 25</t>
         </is>
       </c>
     </row>
@@ -6872,7 +7072,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -6886,7 +7086,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -6922,23 +7122,48 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>12:32:19</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>13:53</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>44</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>14:28</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>116</v>
-      </c>
-      <c r="E29" t="inlineStr">
+      <c r="D30" t="n">
+        <v>79</v>
+      </c>
+      <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4606
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E206"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:09:21</t>
+          <t>Última actualización: 13:36:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 201</t>
+          <t>Total filas: 208</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -4998,7 +4998,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="D187" t="n">
-        <v>31</v>
+        <v>4</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -5023,7 +5023,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="D188" t="n">
-        <v>38</v>
+        <v>11</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -5087,7 +5087,7 @@
         </is>
       </c>
       <c r="D190" t="n">
-        <v>41</v>
+        <v>14</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5162,7 +5162,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>59</v>
+        <v>32</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>81</v>
+        <v>35</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5248,7 +5248,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -5262,7 +5262,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5323,7 +5323,7 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -5337,7 +5337,7 @@
         </is>
       </c>
       <c r="D200" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>92</v>
+        <v>65</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5398,7 +5398,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -5412,7 +5412,7 @@
         </is>
       </c>
       <c r="D203" t="n">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5423,21 +5423,21 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>108</v>
+        <v>79</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>112</v>
+        <v>80</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5478,18 +5478,193 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
+          <t>14:57</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D206" t="n">
+        <v>108</v>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>13:09:21</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D207" t="n">
+        <v>112</v>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>15:05</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D208" t="n">
+        <v>89</v>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
           <t>15:07</t>
         </is>
       </c>
-      <c r="C206" t="inlineStr">
+      <c r="C209" t="inlineStr">
         <is>
           <t>17X38_ROMERO</t>
         </is>
       </c>
-      <c r="D206" t="n">
-        <v>118</v>
-      </c>
-      <c r="E206" t="inlineStr">
+      <c r="D209" t="n">
+        <v>91</v>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D210" t="n">
+        <v>94</v>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>15:11</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D211" t="n">
+        <v>95</v>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D212" t="n">
+        <v>110</v>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>112</v>
+      </c>
+      <c r="E213" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5506,7 +5681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5519,14 +5694,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:09:21</t>
+          <t>Última actualización: 13:36:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 39</t>
         </is>
       </c>
     </row>
@@ -6385,7 +6560,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6399,7 +6574,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -6435,7 +6610,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -6449,7 +6624,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -6460,23 +6635,73 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>14:56</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>80</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>13:09:21</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B43" t="inlineStr">
         <is>
           <t>14:57</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C43" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D42" t="n">
+      <c r="D43" t="n">
         <v>108</v>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>112</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6493,7 +6718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6506,14 +6731,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:09:21</t>
+          <t>Última actualización: 13:36:29</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 25</t>
+          <t>Total filas: 26</t>
         </is>
       </c>
     </row>
@@ -7122,7 +7347,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -7136,7 +7361,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>44</v>
+        <v>17</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -7147,7 +7372,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -7161,11 +7386,36 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>79</v>
+        <v>52</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>15:13</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>97</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4607
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E213"/>
+  <dimension ref="A1:E219"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:36:29</t>
+          <t>Última actualización: 13:54:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 208</t>
+          <t>Total filas: 214</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5123,7 +5123,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -5133,11 +5133,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -5158,11 +5158,11 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -5173,7 +5173,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -5187,7 +5187,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5198,7 +5198,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -5212,7 +5212,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5273,7 +5273,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -5287,7 +5287,7 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,7 +5298,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -5312,7 +5312,7 @@
         </is>
       </c>
       <c r="D199" t="n">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5348,7 +5348,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D201" t="n">
-        <v>65</v>
+        <v>47</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -5387,7 +5387,7 @@
         </is>
       </c>
       <c r="D202" t="n">
-        <v>117</v>
+        <v>53</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,7 +5448,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -5462,7 +5462,7 @@
         </is>
       </c>
       <c r="D205" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>91</v>
+        <v>73</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5583,11 +5583,11 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D210" t="n">
-        <v>94</v>
+        <v>76</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>110</v>
+        <v>77</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5648,23 +5648,173 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D213" t="n">
+        <v>81</v>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D214" t="n">
+        <v>89</v>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D215" t="n">
+        <v>92</v>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D216" t="n">
+        <v>93</v>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
           <t>13:36:29</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
+      <c r="B217" t="inlineStr">
         <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C213" t="inlineStr">
+      <c r="C217" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D213" t="n">
+      <c r="D217" t="n">
         <v>112</v>
       </c>
-      <c r="E213" t="inlineStr">
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D218" t="n">
+        <v>114</v>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>115</v>
+      </c>
+      <c r="E219" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5681,7 +5831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5694,14 +5844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:36:29</t>
+          <t>Última actualización: 13:54:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 39</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -6160,7 +6310,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6170,11 +6320,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -6185,7 +6335,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6195,11 +6345,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6535,7 +6685,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6549,7 +6699,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>97</v>
+        <v>33</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6585,7 +6735,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>12:50:45</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6599,7 +6749,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>117</v>
+        <v>53</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6635,7 +6785,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6649,7 +6799,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -6685,23 +6835,48 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>93</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
           <t>13:36:29</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B45" t="inlineStr">
         <is>
           <t>15:28</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C45" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D45" t="n">
         <v>112</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6718,7 +6893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6731,14 +6906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:36:29</t>
+          <t>Última actualización: 13:54:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 29</t>
         </is>
       </c>
     </row>
@@ -7372,12 +7547,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>13:54</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -7386,7 +7561,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -7397,23 +7572,98 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>14:27</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>33</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>13:36:29</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>14:28</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>52</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>15:12</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>78</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
         <is>
           <t>15:13</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>215A_LA PLATA</t>
         </is>
       </c>
-      <c r="D31" t="n">
+      <c r="D34" t="n">
         <v>97</v>
       </c>
-      <c r="E31" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4608
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E219"/>
+  <dimension ref="A1:E231"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:47</t>
+          <t>Última actualización: 14:09:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 214</t>
+          <t>Total filas: 226</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -5173,21 +5173,21 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>14:11</t>
+          <t>14:09</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D194" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -5203,16 +5203,16 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>14:16</t>
+          <t>14:11</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D195" t="n">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -5223,21 +5223,21 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>14:17</t>
+          <t>14:12</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -5248,21 +5248,21 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>14:25</t>
+          <t>14:16</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D197" t="n">
-        <v>49</v>
+        <v>7</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -5273,21 +5273,21 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>14:26</t>
+          <t>14:17</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D198" t="n">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="E198" t="inlineStr">
         <is>
@@ -5298,21 +5298,21 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>14:27</t>
+          <t>14:25</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D199" t="n">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
@@ -5323,21 +5323,21 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>14:28</t>
+          <t>14:26</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
@@ -5348,21 +5348,21 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>14:41</t>
+          <t>14:27</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D201" t="n">
-        <v>47</v>
+        <v>18</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
@@ -5373,21 +5373,21 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>14:47</t>
+          <t>14:28</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
@@ -5398,21 +5398,21 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>14:48</t>
+          <t>14:40</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="E203" t="inlineStr">
         <is>
@@ -5428,16 +5428,16 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>14:55</t>
+          <t>14:41</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D204" t="n">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5448,21 +5448,21 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>14:56</t>
+          <t>14:47</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D205" t="n">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
@@ -5473,21 +5473,21 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>14:57</t>
+          <t>14:48</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>108</v>
+        <v>72</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,21 +5498,21 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>15:01</t>
+          <t>14:55</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>112</v>
+        <v>46</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,21 +5523,21 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>15:05</t>
+          <t>14:56</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D208" t="n">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5548,21 +5548,21 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>15:07</t>
+          <t>14:57</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D209" t="n">
-        <v>73</v>
+        <v>108</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,12 +5573,12 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:01</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5603,16 +5603,16 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>15:05</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D211" t="n">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
@@ -5623,21 +5623,21 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>15:11</t>
+          <t>15:06</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D212" t="n">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
@@ -5653,16 +5653,16 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:07</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D213" t="n">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,21 +5673,21 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,21 +5698,21 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,21 +5723,21 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:10</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5748,21 +5748,21 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D217" t="n">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5778,16 +5778,16 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D218" t="n">
-        <v>114</v>
+        <v>81</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,23 +5798,323 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>15:18</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D219" t="n">
+        <v>69</v>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D220" t="n">
+        <v>73</v>
+      </c>
+      <c r="E220" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
           <t>13:54:47</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>15:23</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D221" t="n">
+        <v>89</v>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D222" t="n">
+        <v>77</v>
+      </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>15:27</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D223" t="n">
+        <v>78</v>
+      </c>
+      <c r="E223" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>13:36:29</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>15:28</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D224" t="n">
+        <v>112</v>
+      </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>15:47</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D225" t="n">
+        <v>98</v>
+      </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>13:54:47</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>15:48</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D226" t="n">
+        <v>114</v>
+      </c>
+      <c r="E226" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
         <is>
           <t>15:49</t>
         </is>
       </c>
-      <c r="C219" t="inlineStr">
+      <c r="C227" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D219" t="n">
-        <v>115</v>
-      </c>
-      <c r="E219" t="inlineStr">
+      <c r="D227" t="n">
+        <v>100</v>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D228" t="n">
+        <v>107</v>
+      </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D229" t="n">
+        <v>107</v>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D230" t="n">
+        <v>117</v>
+      </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>118</v>
+      </c>
+      <c r="E231" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -5844,7 +6144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:47</t>
+          <t>Última actualización: 14:09:59</t>
         </is>
       </c>
     </row>
@@ -6310,7 +6610,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6320,11 +6620,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -6335,7 +6635,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6345,11 +6645,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -6685,7 +6985,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -6699,7 +6999,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -6735,7 +7035,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -6749,7 +7049,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -6785,7 +7085,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -6799,7 +7099,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>62</v>
+        <v>47</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -6835,7 +7135,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -6849,7 +7149,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -6893,7 +7193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6906,14 +7206,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 13:54:47</t>
+          <t>Última actualización: 14:09:59</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 29</t>
+          <t>Total filas: 30</t>
         </is>
       </c>
     </row>
@@ -7572,7 +7872,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -7586,7 +7886,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -7622,7 +7922,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -7636,7 +7936,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>78</v>
+        <v>63</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -7666,6 +7966,31 @@
       <c r="E34" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>15:52</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>103</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4609
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E231"/>
+  <dimension ref="A1:E242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:09:59</t>
+          <t>Última actualización: 14:33:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 226</t>
+          <t>Total filas: 237</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5423,7 +5423,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -5437,7 +5437,7 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>47</v>
+        <v>8</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
@@ -5473,7 +5473,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -5487,7 +5487,7 @@
         </is>
       </c>
       <c r="D206" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5548,7 +5548,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -5562,7 +5562,7 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>73</v>
+        <v>34</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5748,7 +5748,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -5762,7 +5762,7 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
@@ -5773,12 +5773,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="D218" t="n">
-        <v>81</v>
+        <v>39</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
@@ -5798,12 +5798,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5828,16 +5828,16 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D220" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5848,12 +5848,12 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>77</v>
+        <v>89</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,21 +5898,21 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D223" t="n">
-        <v>78</v>
+        <v>52</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>112</v>
+        <v>77</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5953,16 +5953,16 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>114</v>
+        <v>54</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -5998,21 +5998,21 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,21 +6023,21 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>107</v>
+        <v>68</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6053,16 +6053,16 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>107</v>
+        <v>98</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,21 +6073,21 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>117</v>
+        <v>75</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,18 +6103,293 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
+          <t>15:49</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D231" t="n">
+        <v>100</v>
+      </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D232" t="n">
+        <v>107</v>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>15:56</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D233" t="n">
+        <v>107</v>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>15:57</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D234" t="n">
+        <v>84</v>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>15:59</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D235" t="n">
+        <v>86</v>
+      </c>
+      <c r="E235" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>16:01</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D236" t="n">
+        <v>88</v>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>16:05</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D237" t="n">
+        <v>92</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>16:06</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D238" t="n">
+        <v>117</v>
+      </c>
+      <c r="E238" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
           <t>16:07</t>
         </is>
       </c>
-      <c r="C231" t="inlineStr">
+      <c r="C239" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D231" t="n">
+      <c r="D239" t="n">
         <v>118</v>
       </c>
-      <c r="E231" t="inlineStr">
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D240" t="n">
+        <v>94</v>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D241" t="n">
+        <v>110</v>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>114</v>
+      </c>
+      <c r="E242" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6144,7 +6419,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:09:59</t>
+          <t>Última actualización: 14:33:11</t>
         </is>
       </c>
     </row>
@@ -6610,7 +6885,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6620,11 +6895,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -6635,7 +6910,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6645,11 +6920,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -7060,7 +7335,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7074,7 +7349,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>72</v>
+        <v>15</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -7110,7 +7385,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7124,7 +7399,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>108</v>
+        <v>24</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -7160,7 +7435,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7174,7 +7449,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>112</v>
+        <v>55</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -7193,7 +7468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7206,14 +7481,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:09:59</t>
+          <t>Última actualización: 14:33:11</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 30</t>
+          <t>Total filas: 31</t>
         </is>
       </c>
     </row>
@@ -7947,7 +8222,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -7961,7 +8236,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -7989,6 +8264,31 @@
         <v>103</v>
       </c>
       <c r="E35" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>80</v>
+      </c>
+      <c r="E36" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4610
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E242"/>
+  <dimension ref="A1:E251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:11</t>
+          <t>Última actualización: 14:51:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 237</t>
+          <t>Total filas: 246</t>
         </is>
       </c>
     </row>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -5498,7 +5498,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -5512,7 +5512,7 @@
         </is>
       </c>
       <c r="D207" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
@@ -5523,7 +5523,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5537,7 +5537,7 @@
         </is>
       </c>
       <c r="D208" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E208" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -5587,7 +5587,7 @@
         </is>
       </c>
       <c r="D210" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
@@ -5648,7 +5648,7 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
@@ -5662,7 +5662,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5798,12 +5798,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="D219" t="n">
-        <v>81</v>
+        <v>22</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
@@ -5823,12 +5823,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>15:18</t>
+          <t>15:15</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5837,7 +5837,7 @@
         </is>
       </c>
       <c r="D220" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
@@ -5853,16 +5853,16 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,12 +5873,12 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -5887,7 +5887,7 @@
         </is>
       </c>
       <c r="D222" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>52</v>
+        <v>89</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,21 +5923,21 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D224" t="n">
-        <v>77</v>
+        <v>34</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>78</v>
+        <v>35</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,7 +5973,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -5983,11 +5983,11 @@
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>54</v>
+        <v>36</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6003,16 +6003,16 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6028,16 +6028,16 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6078,16 +6078,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D230" t="n">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6103,16 +6103,16 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,21 +6123,21 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D232" t="n">
-        <v>107</v>
+        <v>57</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6153,16 +6153,16 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6173,21 +6173,21 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>84</v>
+        <v>107</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6228,16 +6228,16 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6253,16 +6253,16 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>117</v>
+        <v>69</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6298,21 +6298,21 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>118</v>
+        <v>88</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6328,16 +6328,16 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,23 +6373,248 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D242" t="n">
+        <v>76</v>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>14:09:59</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D243" t="n">
+        <v>118</v>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>17X38_ROMERO</t>
+        </is>
+      </c>
+      <c r="D244" t="n">
+        <v>76</v>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D245" t="n">
+        <v>79</v>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>16:23</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D246" t="n">
+        <v>92</v>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>16:26</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D247" t="n">
+        <v>95</v>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
           <t>14:33:10</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
+      <c r="B248" t="inlineStr">
         <is>
           <t>16:27</t>
         </is>
       </c>
-      <c r="C242" t="inlineStr">
+      <c r="C248" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D242" t="n">
+      <c r="D248" t="n">
         <v>114</v>
       </c>
-      <c r="E242" t="inlineStr">
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D249" t="n">
+        <v>107</v>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D250" t="n">
+        <v>109</v>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>109</v>
+      </c>
+      <c r="E251" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6419,7 +6644,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:11</t>
+          <t>Última actualización: 14:51:52</t>
         </is>
       </c>
     </row>
@@ -6885,7 +7110,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -6895,11 +7120,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -6910,7 +7135,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -6920,11 +7145,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -7360,7 +7585,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7374,7 +7599,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>47</v>
+        <v>5</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -7410,7 +7635,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7424,7 +7649,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>78</v>
+        <v>36</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7468,7 +7693,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7481,14 +7706,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:33:11</t>
+          <t>Última actualización: 14:51:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 31</t>
+          <t>Total filas: 32</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8422,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -8211,7 +8436,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>63</v>
+        <v>21</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -8247,7 +8472,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -8261,7 +8486,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -8291,6 +8516,31 @@
       <c r="E36" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>14:51:51</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>16:37</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>106</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4611
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E251"/>
+  <dimension ref="A1:E259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:52</t>
+          <t>Última actualización: 15:11:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 246</t>
+          <t>Total filas: 254</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5848,7 +5848,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -5862,7 +5862,7 @@
         </is>
       </c>
       <c r="D221" t="n">
-        <v>69</v>
+        <v>7</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
@@ -5873,21 +5873,21 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15:22</t>
+          <t>15:18</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
-        <v>73</v>
+        <v>7</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
@@ -5898,12 +5898,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>13:54:47</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15:23</t>
+          <t>15:22</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5912,7 +5912,7 @@
         </is>
       </c>
       <c r="D223" t="n">
-        <v>89</v>
+        <v>73</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
@@ -5923,12 +5923,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:54:47</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15:25</t>
+          <t>15:23</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="D224" t="n">
-        <v>34</v>
+        <v>89</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
@@ -5948,21 +5948,21 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15:26</t>
+          <t>15:25</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D225" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
@@ -5973,21 +5973,21 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15:27</t>
+          <t>15:26</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D226" t="n">
-        <v>36</v>
+        <v>15</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
@@ -6023,12 +6023,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15:28</t>
+          <t>15:27</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -6037,7 +6037,7 @@
         </is>
       </c>
       <c r="D228" t="n">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6048,21 +6048,21 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15:40</t>
+          <t>15:28</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D229" t="n">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E229" t="inlineStr">
         <is>
@@ -6073,12 +6073,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15:41</t>
+          <t>15:40</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="D230" t="n">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
@@ -6098,21 +6098,21 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15:47</t>
+          <t>15:41</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D231" t="n">
-        <v>98</v>
+        <v>30</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
@@ -6123,12 +6123,12 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15:48</t>
+          <t>15:47</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -6137,7 +6137,7 @@
         </is>
       </c>
       <c r="D232" t="n">
-        <v>57</v>
+        <v>98</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
@@ -6148,21 +6148,21 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15:49</t>
+          <t>15:48</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D233" t="n">
-        <v>100</v>
+        <v>37</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
@@ -6178,16 +6178,16 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:49</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D234" t="n">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
@@ -6198,21 +6198,21 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>15:56</t>
+          <t>15:55</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D235" t="n">
-        <v>65</v>
+        <v>44</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
@@ -6223,12 +6223,12 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>15:57</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="D236" t="n">
-        <v>84</v>
+        <v>45</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
@@ -6248,21 +6248,21 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>15:59</t>
+          <t>15:56</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D237" t="n">
-        <v>86</v>
+        <v>45</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
@@ -6273,21 +6273,21 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>15:57</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D238" t="n">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -6303,16 +6303,16 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>16:01</t>
+          <t>15:59</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D239" t="n">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
@@ -6323,21 +6323,21 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>16:05</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>92</v>
+        <v>69</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
@@ -6348,21 +6348,21 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>16:06</t>
+          <t>16:01</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D241" t="n">
-        <v>117</v>
+        <v>88</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
@@ -6373,21 +6373,21 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:05</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
@@ -6403,16 +6403,16 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>16:07</t>
+          <t>16:06</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D243" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6437,7 +6437,7 @@
         </is>
       </c>
       <c r="D244" t="n">
-        <v>76</v>
+        <v>56</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,21 +6448,21 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>79</v>
+        <v>56</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,21 +6473,21 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:07</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>92</v>
+        <v>118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6503,16 +6503,16 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D247" t="n">
-        <v>95</v>
+        <v>79</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,21 +6523,21 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D248" t="n">
-        <v>114</v>
+        <v>60</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6548,21 +6548,21 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>109</v>
+        <v>75</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,23 +6598,223 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
+          <t>14:33:10</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>16:27</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D251" t="n">
+        <v>114</v>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D252" t="n">
+        <v>87</v>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D253" t="n">
+        <v>89</v>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
           <t>14:51:51</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
+      <c r="B254" t="inlineStr">
         <is>
           <t>16:40</t>
         </is>
       </c>
-      <c r="C251" t="inlineStr">
+      <c r="C254" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D251" t="n">
+      <c r="D254" t="n">
         <v>109</v>
       </c>
-      <c r="E251" t="inlineStr">
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D255" t="n">
+        <v>90</v>
+      </c>
+      <c r="E255" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>16:41</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D256" t="n">
+        <v>90</v>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D257" t="n">
+        <v>102</v>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D258" t="n">
+        <v>105</v>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>116</v>
+      </c>
+      <c r="E259" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6631,7 +6831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6644,14 +6844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:52</t>
+          <t>Última actualización: 15:11:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -7635,7 +7835,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7649,7 +7849,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>36</v>
+        <v>16</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -7677,6 +7877,31 @@
         <v>55</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>17:07</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>116</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7693,7 +7918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7706,14 +7931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 14:51:52</t>
+          <t>Última actualización: 15:11:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 32</t>
+          <t>Total filas: 34</t>
         </is>
       </c>
     </row>
@@ -8422,12 +8647,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15:12</t>
+          <t>15:11</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -8436,7 +8661,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -8447,12 +8672,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15:13</t>
+          <t>15:12</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -8461,7 +8686,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -8472,37 +8697,37 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>15:52</t>
+          <t>15:13</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>215C_LA PLATA</t>
+          <t>215A_LA PLATA</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>61</v>
+        <v>40</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>L6203</t>
+          <t>L6173</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15:53</t>
+          <t>15:52</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -8511,7 +8736,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -8522,25 +8747,75 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>15:53</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>80</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>16:37</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-40 Y 115</t>
         </is>
       </c>
-      <c r="D37" t="n">
-        <v>106</v>
-      </c>
-      <c r="E37" t="inlineStr">
+      <c r="D38" t="n">
+        <v>86</v>
+      </c>
+      <c r="E38" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>15:11:48</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>17:02</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>111</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4612
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -432,7 +432,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:48</t>
+          <t>Última actualización: 15:49:06</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6708,7 +6708,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -6844,7 +6844,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:48</t>
+          <t>Última actualización: 15:49:06</t>
         </is>
       </c>
     </row>
@@ -7918,7 +7918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7931,14 +7931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:11:48</t>
+          <t>Última actualización: 15:49:06</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 34</t>
+          <t>Total filas: 36</t>
         </is>
       </c>
     </row>
@@ -8747,7 +8747,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:49:06</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8761,7 +8761,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8797,23 +8797,73 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>15:49:06</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>16:38</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>49</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>15:11:48</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B40" t="inlineStr">
         <is>
           <t>17:02</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C40" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D39" t="n">
+      <c r="D40" t="n">
         <v>111</v>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>15:49:06</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>17:03</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>74</v>
+      </c>
+      <c r="E41" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4613
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E259"/>
+  <dimension ref="A1:E271"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:06</t>
+          <t>Última actualización: 16:09:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 254</t>
+          <t>Total filas: 266</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6498,12 +6498,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>16:10</t>
+          <t>16:09</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="D247" t="n">
-        <v>79</v>
+        <v>0</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
@@ -6523,12 +6523,12 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>16:11</t>
+          <t>16:10</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
@@ -6537,7 +6537,7 @@
         </is>
       </c>
       <c r="D248" t="n">
-        <v>60</v>
+        <v>79</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
@@ -6553,16 +6553,16 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>16:23</t>
+          <t>16:11</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>83_ALUAR</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D249" t="n">
-        <v>72</v>
+        <v>60</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
@@ -6573,21 +6573,21 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>16:26</t>
+          <t>16:23</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>83_ALUAR</t>
         </is>
       </c>
       <c r="D250" t="n">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
@@ -6598,21 +6598,21 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>16:27</t>
+          <t>16:25</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D251" t="n">
-        <v>114</v>
+        <v>16</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
@@ -6623,21 +6623,21 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>16:38</t>
+          <t>16:26</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D252" t="n">
-        <v>87</v>
+        <v>17</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
@@ -6648,21 +6648,21 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:27</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D253" t="n">
-        <v>89</v>
+        <v>114</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
@@ -6673,21 +6673,21 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>16:40</t>
+          <t>16:38</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D254" t="n">
-        <v>109</v>
+        <v>29</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,21 +6698,21 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>90</v>
+        <v>109</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,21 +6723,21 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>16:41</t>
+          <t>16:40</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>90</v>
+        <v>31</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6748,21 +6748,21 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>102</v>
+        <v>32</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,21 +6773,21 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:41</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>105</v>
+        <v>32</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,23 +6798,323 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>16:53</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D259" t="n">
+        <v>44</v>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>16:55</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D260" t="n">
+        <v>46</v>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D261" t="n">
+        <v>47</v>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
           <t>15:11:48</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr">
+      <c r="B262" t="inlineStr">
         <is>
           <t>17:07</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr">
+      <c r="C262" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D259" t="n">
+      <c r="D262" t="n">
         <v>116</v>
       </c>
-      <c r="E259" t="inlineStr">
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D263" t="n">
+        <v>59</v>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>17:22</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D264" t="n">
+        <v>73</v>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D265" t="n">
+        <v>83</v>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>17:38</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>89</v>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>17:41</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>92</v>
+      </c>
+      <c r="E267" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>17:46</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>97</v>
+      </c>
+      <c r="E268" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>101</v>
+      </c>
+      <c r="E269" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>104</v>
+      </c>
+      <c r="E270" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>18:05</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>116</v>
+      </c>
+      <c r="E271" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -6831,7 +7131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6844,14 +7144,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:06</t>
+          <t>Última actualización: 16:09:25</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -7310,7 +7610,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7320,11 +7620,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -7335,7 +7635,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7345,11 +7645,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -7902,6 +8202,81 @@
         <v>116</v>
       </c>
       <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>17:08</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>59</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>17:32</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>83</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>16:09:25</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>104</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7931,7 +8306,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 15:49:06</t>
+          <t>Última actualización: 16:09:25</t>
         </is>
       </c>
     </row>
@@ -8797,7 +9172,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>15:49:06</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -8811,7 +9186,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>49</v>
+        <v>29</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8847,7 +9222,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>15:49:06</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8861,7 +9236,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>74</v>
+        <v>54</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4614
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E271"/>
+  <dimension ref="A1:E279"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:25</t>
+          <t>Última actualización: 16:31:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 266</t>
+          <t>Total filas: 274</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6673,7 +6673,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -6687,7 +6687,7 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>109</v>
+        <v>9</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>31</v>
+        <v>109</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6758,7 +6758,7 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6798,21 +6798,21 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>16:53</t>
+          <t>16:43</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D259" t="n">
-        <v>44</v>
+        <v>12</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
@@ -6823,21 +6823,21 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>16:55</t>
+          <t>16:53</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D260" t="n">
-        <v>46</v>
+        <v>22</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,21 +6848,21 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>16:56</t>
+          <t>16:55</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D261" t="n">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,21 +6873,21 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>17:07</t>
+          <t>16:56</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D262" t="n">
-        <v>116</v>
+        <v>25</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6898,12 +6898,12 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>17:08</t>
+          <t>17:07</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -6912,7 +6912,7 @@
         </is>
       </c>
       <c r="D263" t="n">
-        <v>59</v>
+        <v>116</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -6923,21 +6923,21 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:08</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D264" t="n">
-        <v>73</v>
+        <v>37</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>83</v>
+        <v>51</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>89</v>
+        <v>54</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>92</v>
+        <v>61</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>97</v>
+        <v>67</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7078,16 +7078,16 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
-        <v>104</v>
+        <v>92</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7103,18 +7103,218 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
+          <t>17:46</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>97</v>
+      </c>
+      <c r="E271" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>79</v>
+      </c>
+      <c r="E272" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>82</v>
+      </c>
+      <c r="E273" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>82</v>
+      </c>
+      <c r="E274" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
           <t>18:05</t>
         </is>
       </c>
-      <c r="C271" t="inlineStr">
+      <c r="C275" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D271" t="n">
-        <v>116</v>
-      </c>
-      <c r="E271" t="inlineStr">
+      <c r="D275" t="n">
+        <v>94</v>
+      </c>
+      <c r="E275" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>97</v>
+      </c>
+      <c r="E276" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>99</v>
+      </c>
+      <c r="E277" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>109</v>
+      </c>
+      <c r="E278" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>112</v>
+      </c>
+      <c r="E279" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7131,7 +7331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7144,14 +7344,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:25</t>
+          <t>Última actualización: 16:31:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 45</t>
         </is>
       </c>
     </row>
@@ -8210,7 +8410,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8224,7 +8424,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8235,7 +8435,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8249,7 +8449,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>83</v>
+        <v>61</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8260,7 +8460,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8274,9 +8474,34 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>112</v>
+      </c>
+      <c r="E50" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8293,7 +8518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8306,14 +8531,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:09:25</t>
+          <t>Última actualización: 16:31:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 36</t>
+          <t>Total filas: 37</t>
         </is>
       </c>
     </row>
@@ -9172,7 +9397,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -9186,7 +9411,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>29</v>
+        <v>7</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -9222,7 +9447,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9236,9 +9461,34 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="E41" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>16:31:31</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>119</v>
+      </c>
+      <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4615
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E279"/>
+  <dimension ref="A1:E284"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:31</t>
+          <t>Última actualización: 16:50:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 274</t>
+          <t>Total filas: 279</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>109</v>
+        <v>9</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -6823,7 +6823,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="D260" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
@@ -6848,7 +6848,7 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
@@ -6862,7 +6862,7 @@
         </is>
       </c>
       <c r="D261" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
@@ -6873,7 +6873,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
@@ -6887,7 +6887,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
@@ -6923,7 +6923,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
@@ -6937,7 +6937,7 @@
         </is>
       </c>
       <c r="D264" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
@@ -6948,7 +6948,7 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
@@ -6962,7 +6962,7 @@
         </is>
       </c>
       <c r="D265" t="n">
-        <v>51</v>
+        <v>32</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,7 +6973,7 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
@@ -6987,7 +6987,7 @@
         </is>
       </c>
       <c r="D266" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,7 +6998,7 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
@@ -7012,7 +7012,7 @@
         </is>
       </c>
       <c r="D267" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>67</v>
+        <v>46</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,12 +7073,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7103,16 +7103,16 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7203,16 +7203,16 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>97</v>
+        <v>63</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>99</v>
+        <v>75</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>109</v>
+        <v>78</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,23 +7298,148 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
+          <t>18:10</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>80</v>
+      </c>
+      <c r="E279" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>16:50:26</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>18:20</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>90</v>
+      </c>
+      <c r="E280" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>16:50:26</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C279" t="inlineStr">
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>93</v>
+      </c>
+      <c r="E281" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>16:50:26</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D279" t="n">
-        <v>112</v>
-      </c>
-      <c r="E279" t="inlineStr">
+      <c r="D282" t="n">
+        <v>93</v>
+      </c>
+      <c r="E282" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>16:50:26</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>105</v>
+      </c>
+      <c r="E283" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>16:50:26</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>15X38_ABASTO</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>107</v>
+      </c>
+      <c r="E284" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7344,7 +7469,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:31</t>
+          <t>Última actualización: 16:50:26</t>
         </is>
       </c>
     </row>
@@ -8410,7 +8535,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -8424,7 +8549,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>37</v>
+        <v>18</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -8435,7 +8560,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -8449,7 +8574,7 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8460,7 +8585,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -8474,7 +8599,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>82</v>
+        <v>63</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8485,7 +8610,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8499,7 +8624,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8531,7 +8656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:31:31</t>
+          <t>Última actualización: 16:50:26</t>
         </is>
       </c>
     </row>
@@ -9447,7 +9572,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -9461,7 +9586,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -9472,7 +9597,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9486,7 +9611,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4616
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E284"/>
+  <dimension ref="A1:E292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:26</t>
+          <t>Última actualización: 17:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 279</t>
+          <t>Total filas: 287</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -6948,21 +6948,21 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>17:22</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
@@ -6973,21 +6973,21 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>17:25</t>
+          <t>17:22</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D266" t="n">
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
@@ -6998,21 +6998,21 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:25</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D267" t="n">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
@@ -7023,21 +7023,21 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>17:36</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D268" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
@@ -7048,21 +7048,21 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:35</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D269" t="n">
-        <v>48</v>
+        <v>26</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
@@ -7073,12 +7073,12 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>68</v>
+        <v>46</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,12 +7098,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -7112,7 +7112,7 @@
         </is>
       </c>
       <c r="D271" t="n">
-        <v>92</v>
+        <v>28</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7123,21 +7123,21 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>97</v>
+        <v>29</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,21 +7173,21 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D274" t="n">
-        <v>62</v>
+        <v>92</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7198,12 +7198,12 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
@@ -7212,7 +7212,7 @@
         </is>
       </c>
       <c r="D275" t="n">
-        <v>82</v>
+        <v>97</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>63</v>
+        <v>41</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7253,16 +7253,16 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>75</v>
+        <v>62</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,21 +7273,21 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D278" t="n">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,21 +7298,21 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>90</v>
+        <v>56</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>93</v>
+        <v>59</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>105</v>
+        <v>71</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7428,18 +7428,218 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D284" t="n">
+        <v>93</v>
+      </c>
+      <c r="E284" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>74</v>
+      </c>
+      <c r="E285" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>75</v>
+      </c>
+      <c r="E286" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>77</v>
+      </c>
+      <c r="E287" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>18:35</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>86</v>
+      </c>
+      <c r="E288" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
           <t>18:37</t>
         </is>
       </c>
-      <c r="C284" t="inlineStr">
+      <c r="C289" t="inlineStr">
         <is>
           <t>15X38_ABASTO</t>
         </is>
       </c>
-      <c r="D284" t="n">
-        <v>107</v>
-      </c>
-      <c r="E284" t="inlineStr">
+      <c r="D289" t="n">
+        <v>88</v>
+      </c>
+      <c r="E289" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>104</v>
+      </c>
+      <c r="E290" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>116</v>
+      </c>
+      <c r="E291" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>119</v>
+      </c>
+      <c r="E292" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7456,7 +7656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7469,14 +7669,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:26</t>
+          <t>Última actualización: 17:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 45</t>
+          <t>Total filas: 47</t>
         </is>
       </c>
     </row>
@@ -7935,7 +8135,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7945,11 +8145,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -7960,7 +8160,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -7970,11 +8170,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -8560,21 +8760,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>17:32</t>
+          <t>17:09</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -8585,21 +8785,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:32</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>63</v>
+        <v>23</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -8610,23 +8810,73 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>17:53</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>44</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
           <t>18:23</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C51" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D50" t="n">
-        <v>93</v>
-      </c>
-      <c r="E50" t="inlineStr">
+      <c r="D51" t="n">
+        <v>74</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>119</v>
+      </c>
+      <c r="E52" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8643,7 +8893,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8656,14 +8906,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 16:50:26</t>
+          <t>Última actualización: 17:09:21</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 37</t>
+          <t>Total filas: 38</t>
         </is>
       </c>
     </row>
@@ -9597,7 +9847,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9611,11 +9861,36 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>100</v>
+        <v>81</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:09:21</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>19:02</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>113</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4617
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E292"/>
+  <dimension ref="A1:E298"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:09:21</t>
+          <t>Última actualización: 17:35:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 287</t>
+          <t>Total filas: 293</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -7073,7 +7073,7 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
@@ -7087,7 +7087,7 @@
         </is>
       </c>
       <c r="D270" t="n">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
@@ -7098,21 +7098,21 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>17:37</t>
+          <t>17:36</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
-        <v>28</v>
+        <v>1</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
@@ -7128,16 +7128,16 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>17:38</t>
+          <t>17:37</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D272" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
@@ -7148,21 +7148,21 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>17:39</t>
+          <t>17:38</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D273" t="n">
-        <v>68</v>
+        <v>3</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
@@ -7173,12 +7173,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>17:41</t>
+          <t>17:39</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -7187,7 +7187,7 @@
         </is>
       </c>
       <c r="D274" t="n">
-        <v>92</v>
+        <v>68</v>
       </c>
       <c r="E274" t="inlineStr">
         <is>
@@ -7203,16 +7203,16 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>17:46</t>
+          <t>17:41</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D275" t="n">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
@@ -7223,21 +7223,21 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>17:50</t>
+          <t>17:46</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D276" t="n">
-        <v>41</v>
+        <v>97</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
@@ -7248,21 +7248,21 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>17:52</t>
+          <t>17:50</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D277" t="n">
-        <v>62</v>
+        <v>15</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
@@ -7273,12 +7273,12 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>17:53</t>
+          <t>17:52</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
@@ -7287,7 +7287,7 @@
         </is>
       </c>
       <c r="D278" t="n">
-        <v>82</v>
+        <v>62</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,21 +7323,21 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:53</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>56</v>
+        <v>82</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>61</v>
+        <v>33</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>71</v>
+        <v>35</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>93</v>
+        <v>45</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,7 +7448,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
@@ -7462,7 +7462,7 @@
         </is>
       </c>
       <c r="D285" t="n">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7503,16 +7503,16 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>88</v>
+        <v>51</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>104</v>
+        <v>60</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>116</v>
+        <v>62</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,23 +7623,173 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
+          <t>18:53</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>78</v>
+      </c>
+      <c r="E292" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>80</v>
+      </c>
+      <c r="E293" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>90</v>
+      </c>
+      <c r="E294" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
           <t>19:08</t>
         </is>
       </c>
-      <c r="C292" t="inlineStr">
+      <c r="C295" t="inlineStr">
         <is>
           <t>215_EL PELIGRO</t>
         </is>
       </c>
-      <c r="D292" t="n">
-        <v>119</v>
-      </c>
-      <c r="E292" t="inlineStr">
+      <c r="D295" t="n">
+        <v>93</v>
+      </c>
+      <c r="E295" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>101</v>
+      </c>
+      <c r="E296" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>106</v>
+      </c>
+      <c r="E297" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>108</v>
+      </c>
+      <c r="E298" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7656,7 +7806,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7669,14 +7819,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:09:21</t>
+          <t>Última actualización: 17:35:27</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 47</t>
+          <t>Total filas: 48</t>
         </is>
       </c>
     </row>
@@ -8810,7 +8960,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8824,7 +8974,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8835,7 +8985,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8849,7 +8999,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -8860,7 +9010,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -8874,9 +9024,34 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>119</v>
+        <v>93</v>
       </c>
       <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>17:35:27</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>108</v>
+      </c>
+      <c r="E53" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8906,7 +9081,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:09:21</t>
+          <t>Última actualización: 17:35:27</t>
         </is>
       </c>
     </row>
@@ -9847,7 +10022,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -9861,7 +10036,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>81</v>
+        <v>55</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -9872,7 +10047,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -9886,7 +10061,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4618
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E298"/>
+  <dimension ref="A1:E306"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:27</t>
+          <t>Última actualización: 17:53:20</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 293</t>
+          <t>Total filas: 301</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7312,7 +7312,7 @@
         </is>
       </c>
       <c r="D279" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7348,21 +7348,21 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>18:05</t>
+          <t>17:54</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D281" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -7373,21 +7373,21 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>18:08</t>
+          <t>18:05</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D282" t="n">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
@@ -7398,21 +7398,21 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>18:10</t>
+          <t>18:08</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D283" t="n">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
@@ -7423,21 +7423,21 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:10</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D284" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,12 +7473,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -7487,7 +7487,7 @@
         </is>
       </c>
       <c r="D286" t="n">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>75</v>
+        <v>30</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,21 +7523,21 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>50</v>
+        <v>93</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,21 +7573,21 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D290" t="n">
-        <v>60</v>
+        <v>32</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7603,16 +7603,16 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>78</v>
+        <v>42</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>80</v>
+        <v>44</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>90</v>
+        <v>57</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>93</v>
+        <v>60</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>101</v>
+        <v>62</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>106</v>
+        <v>72</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,23 +7773,223 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>19:08</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>215_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>75</v>
+      </c>
+      <c r="E298" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
           <t>17:35:27</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr">
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>19:16</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>101</v>
+      </c>
+      <c r="E299" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>88</v>
+      </c>
+      <c r="E300" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>19:22</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>89</v>
+      </c>
+      <c r="E301" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
         <is>
           <t>19:23</t>
         </is>
       </c>
-      <c r="C298" t="inlineStr">
+      <c r="C302" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D298" t="n">
-        <v>108</v>
-      </c>
-      <c r="E298" t="inlineStr">
+      <c r="D302" t="n">
+        <v>90</v>
+      </c>
+      <c r="E302" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>19:34</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>101</v>
+      </c>
+      <c r="E303" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>107</v>
+      </c>
+      <c r="E304" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>110</v>
+      </c>
+      <c r="E305" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>113</v>
+      </c>
+      <c r="E306" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -7819,7 +8019,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:27</t>
+          <t>Última actualización: 17:53:20</t>
         </is>
       </c>
     </row>
@@ -8960,7 +9160,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -8974,7 +9174,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -8985,7 +9185,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -8999,7 +9199,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9010,7 +9210,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9024,7 +9224,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9035,7 +9235,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9049,7 +9249,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>108</v>
+        <v>90</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9081,7 +9281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:35:27</t>
+          <t>Última actualización: 17:53:20</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10222,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -10036,7 +10236,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -10047,7 +10247,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -10061,7 +10261,7 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>87</v>
+        <v>69</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4619
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E306"/>
+  <dimension ref="A1:E311"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:20</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 301</t>
+          <t>Total filas: 306</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -7423,7 +7423,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -7437,7 +7437,7 @@
         </is>
       </c>
       <c r="D284" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
@@ -7448,21 +7448,21 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>18:20</t>
+          <t>18:11</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D285" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
@@ -7473,21 +7473,21 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>18:21</t>
+          <t>18:20</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D286" t="n">
-        <v>28</v>
+        <v>10</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
@@ -7498,21 +7498,21 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>18:23</t>
+          <t>18:21</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D287" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,21 +7548,21 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>17:09:21</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>18:24</t>
+          <t>18:23</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>75</v>
+        <v>93</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7573,12 +7573,12 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>17:09:21</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>18:25</t>
+          <t>18:24</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
@@ -7587,7 +7587,7 @@
         </is>
       </c>
       <c r="D290" t="n">
-        <v>32</v>
+        <v>75</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
@@ -7598,21 +7598,21 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>18:26</t>
+          <t>18:25</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D291" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
@@ -7623,21 +7623,21 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>18:35</t>
+          <t>18:26</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D292" t="n">
-        <v>42</v>
+        <v>51</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
@@ -7648,21 +7648,21 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,21 +7673,21 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>101</v>
+        <v>58</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>89</v>
+        <v>71</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7878,16 +7878,16 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>19:34</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>107</v>
+        <v>79</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7953,16 +7953,16 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,23 +7973,148 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>90</v>
+      </c>
+      <c r="E306" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>91</v>
+      </c>
+      <c r="E307" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>93</v>
+      </c>
+      <c r="E308" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
           <t>17:53:20</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr">
+      <c r="B309" t="inlineStr">
         <is>
           <t>19:46</t>
         </is>
       </c>
-      <c r="C306" t="inlineStr">
+      <c r="C309" t="inlineStr">
         <is>
           <t>225_GOMEZ</t>
         </is>
       </c>
-      <c r="D306" t="n">
+      <c r="D309" t="n">
         <v>113</v>
       </c>
-      <c r="E306" t="inlineStr">
+      <c r="E309" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>101</v>
+      </c>
+      <c r="E310" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>112</v>
+      </c>
+      <c r="E311" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8019,7 +8144,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:20</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
@@ -9185,7 +9310,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -9199,7 +9324,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -9210,7 +9335,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9224,7 +9349,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>75</v>
+        <v>58</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9235,7 +9360,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9249,7 +9374,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>90</v>
+        <v>73</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9268,7 +9393,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9281,14 +9406,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 17:53:20</t>
+          <t>Última actualización: 18:10:26</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 38</t>
+          <t>Total filas: 40</t>
         </is>
       </c>
     </row>
@@ -10247,25 +10372,75 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>21</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
           <t>19:02</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C44" t="inlineStr">
         <is>
           <t>215B_LP-P MOR-1 Y 57</t>
         </is>
       </c>
-      <c r="D43" t="n">
-        <v>69</v>
-      </c>
-      <c r="E43" t="inlineStr">
+      <c r="D44" t="n">
+        <v>52</v>
+      </c>
+      <c r="E44" t="inlineStr">
         <is>
           <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>18:10:26</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>112</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4620
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E311"/>
+  <dimension ref="A1:E321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:35:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 306</t>
+          <t>Total filas: 316</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7678,16 +7678,16 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>18:37</t>
+          <t>18:35</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7698,21 +7698,21 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>18:50</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
@@ -7723,21 +7723,21 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:37</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
-        <v>43</v>
+        <v>2</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
@@ -7748,21 +7748,21 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:50</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D297" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
@@ -7773,21 +7773,21 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D298" t="n">
-        <v>55</v>
+        <v>18</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7803,16 +7803,16 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7848,21 +7848,21 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>71</v>
+        <v>33</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,12 +7923,12 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7937,7 +7937,7 @@
         </is>
       </c>
       <c r="D304" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>19:34</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>101</v>
+        <v>48</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>90</v>
+        <v>51</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8003,16 +8003,16 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8053,16 +8053,16 @@
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>101</v>
+        <v>65</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,23 +8098,273 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>19:41</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D311" t="n">
+        <v>66</v>
+      </c>
+      <c r="E311" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>19:43</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>81_EL PELIGRO</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>68</v>
+      </c>
+      <c r="E312" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>17:53:20</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>19:46</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>225_GOMEZ</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>113</v>
+      </c>
+      <c r="E313" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
           <t>18:10:26</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>19:51</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>101</v>
+      </c>
+      <c r="E314" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>19:59</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>84</v>
+      </c>
+      <c r="E315" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
         <is>
           <t>20:02</t>
         </is>
       </c>
-      <c r="C311" t="inlineStr">
+      <c r="C316" t="inlineStr">
         <is>
           <t>14_ABASTO</t>
         </is>
       </c>
-      <c r="D311" t="n">
-        <v>112</v>
-      </c>
-      <c r="E311" t="inlineStr">
+      <c r="D316" t="n">
+        <v>87</v>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>88</v>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>100</v>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>101</v>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>107</v>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>110</v>
+      </c>
+      <c r="E321" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8131,7 +8381,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8144,14 +8394,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:35:31</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 48</t>
+          <t>Total filas: 49</t>
         </is>
       </c>
     </row>
@@ -9335,7 +9585,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9349,7 +9599,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>58</v>
+        <v>33</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9360,7 +9610,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9374,9 +9624,34 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>73</v>
+        <v>48</v>
       </c>
       <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>88</v>
+      </c>
+      <c r="E54" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9406,7 +9681,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:10:26</t>
+          <t>Última actualización: 18:35:31</t>
         </is>
       </c>
     </row>
@@ -10397,7 +10672,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10411,7 +10686,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -10422,7 +10697,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10436,7 +10711,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>112</v>
+        <v>87</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4621
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E321"/>
+  <dimension ref="A1:E331"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:31</t>
+          <t>Última actualización: 18:51:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 316</t>
+          <t>Total filas: 326</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6458,7 +6458,7 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D245" t="n">
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7773,12 +7773,12 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>18:53</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
@@ -7787,7 +7787,7 @@
         </is>
       </c>
       <c r="D298" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
@@ -7798,21 +7798,21 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>18:55</t>
+          <t>18:51</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D299" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
@@ -7823,21 +7823,21 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>19:05</t>
+          <t>18:52</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D300" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
@@ -7853,16 +7853,16 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>19:08</t>
+          <t>18:53</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="E301" t="inlineStr">
         <is>
@@ -7873,21 +7873,21 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>18:55</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D302" t="n">
-        <v>101</v>
+        <v>45</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
@@ -7898,21 +7898,21 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:05</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D303" t="n">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
@@ -7923,21 +7923,21 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:08</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D304" t="n">
-        <v>89</v>
+        <v>17</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,21 +7973,21 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D306" t="n">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -7998,21 +7998,21 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>79</v>
+        <v>30</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,12 +8023,12 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -8037,7 +8037,7 @@
         </is>
       </c>
       <c r="D308" t="n">
-        <v>58</v>
+        <v>89</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>19:34</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8073,21 +8073,21 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8103,16 +8103,16 @@
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>66</v>
+        <v>51</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>113</v>
+        <v>58</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,12 +8173,12 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>84</v>
+        <v>49</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>87</v>
+        <v>50</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8273,21 +8273,21 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,17 +8298,17 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D319" t="n">
@@ -8328,16 +8328,16 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>107</v>
+        <v>84</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,23 +8348,273 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>70</v>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>20:01</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>70</v>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>71</v>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>72</v>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
           <t>18:35:31</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>100</v>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>101</v>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D327" t="n">
+        <v>91</v>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
         <is>
           <t>20:25</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr">
+      <c r="C328" t="inlineStr">
         <is>
           <t>15_ABASTO</t>
         </is>
       </c>
-      <c r="D321" t="n">
+      <c r="D328" t="n">
+        <v>94</v>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D329" t="n">
+        <v>101</v>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D330" t="n">
         <v>110</v>
       </c>
-      <c r="E321" t="inlineStr">
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>114</v>
+      </c>
+      <c r="E331" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8381,7 +8631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E54"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8394,14 +8644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:31</t>
+          <t>Última actualización: 18:51:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 49</t>
+          <t>Total filas: 50</t>
         </is>
       </c>
     </row>
@@ -9585,7 +9835,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -9599,7 +9849,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -9610,7 +9860,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -9624,7 +9874,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9635,7 +9885,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -9649,9 +9899,34 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>110</v>
+      </c>
+      <c r="E55" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9668,7 +9943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9681,14 +9956,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:35:31</t>
+          <t>Última actualización: 18:51:28</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 40</t>
+          <t>Total filas: 41</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10947,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -10686,7 +10961,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -10697,7 +10972,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10711,9 +10986,34 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>87</v>
+        <v>71</v>
       </c>
       <c r="E45" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>111</v>
+      </c>
+      <c r="E46" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4622
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E331"/>
+  <dimension ref="A1:E342"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:28</t>
+          <t>Última actualización: 19:09:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 326</t>
+          <t>Total filas: 337</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -6423,7 +6423,7 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
@@ -6433,11 +6433,11 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7948,21 +7948,21 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>19:14</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D305" t="n">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
@@ -7973,12 +7973,12 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>19:16</t>
+          <t>19:10</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7987,7 +7987,7 @@
         </is>
       </c>
       <c r="D306" t="n">
-        <v>101</v>
+        <v>1</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
@@ -8003,16 +8003,16 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>19:21</t>
+          <t>19:14</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D307" t="n">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
@@ -8023,21 +8023,21 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>19:22</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,21 +8048,21 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:16</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8078,16 +8078,16 @@
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>19:25</t>
+          <t>19:21</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D310" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
@@ -8098,21 +8098,21 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>19:26</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>51</v>
+        <v>89</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,21 +8123,21 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>19:29</t>
+          <t>19:22</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>79</v>
+        <v>13</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8148,21 +8148,21 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>19:33</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D313" t="n">
-        <v>58</v>
+        <v>14</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
@@ -8173,21 +8173,21 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>19:34</t>
+          <t>19:25</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D314" t="n">
-        <v>101</v>
+        <v>16</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
@@ -8198,21 +8198,21 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>19:40</t>
+          <t>19:26</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D315" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
@@ -8223,21 +8223,21 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>19:41</t>
+          <t>19:29</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D316" t="n">
-        <v>50</v>
+        <v>79</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
@@ -8248,21 +8248,21 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>19:43</t>
+          <t>19:33</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D317" t="n">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
@@ -8278,16 +8278,16 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>19:46</t>
+          <t>19:34</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D318" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
@@ -8298,21 +8298,21 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>19:51</t>
+          <t>19:40</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D319" t="n">
-        <v>101</v>
+        <v>31</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,21 +8323,21 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:41</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D320" t="n">
-        <v>84</v>
+        <v>32</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,21 +8348,21 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:43</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D321" t="n">
-        <v>70</v>
+        <v>34</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8373,21 +8373,21 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:46</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D322" t="n">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
@@ -8398,21 +8398,21 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>19:51</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D323" t="n">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
@@ -8423,21 +8423,21 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D324" t="n">
-        <v>72</v>
+        <v>84</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,21 +8448,21 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D325" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,12 +8473,12 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -8487,7 +8487,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>101</v>
+        <v>70</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8503,16 +8503,16 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>91</v>
+        <v>71</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>94</v>
+        <v>54</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>110</v>
+        <v>54</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,23 +8598,298 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D331" t="n">
+        <v>100</v>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>18:35:31</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>20:16</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D332" t="n">
+        <v>101</v>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
           <t>18:51:28</t>
         </is>
       </c>
-      <c r="B331" t="inlineStr">
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>20:22</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D333" t="n">
+        <v>91</v>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>20:23</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D334" t="n">
+        <v>74</v>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>20:25</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D335" t="n">
+        <v>76</v>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>20:32</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D336" t="n">
+        <v>101</v>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>18:51:28</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D337" t="n">
+        <v>110</v>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D338" t="n">
+        <v>93</v>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
         <is>
           <t>20:45</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr">
+      <c r="C339" t="inlineStr">
         <is>
           <t>17_ROMERO</t>
         </is>
       </c>
-      <c r="D331" t="n">
+      <c r="D339" t="n">
+        <v>96</v>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>20:50</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D340" t="n">
+        <v>101</v>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D341" t="n">
+        <v>113</v>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
         <v>114</v>
       </c>
-      <c r="E331" t="inlineStr">
+      <c r="E342" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8631,7 +8906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E55"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8644,14 +8919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:28</t>
+          <t>Última actualización: 19:09:10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 50</t>
+          <t>Total filas: 52</t>
         </is>
       </c>
     </row>
@@ -9860,21 +10135,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>19:23</t>
+          <t>19:09</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9885,12 +10160,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>19:23</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -9899,7 +10174,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>72</v>
+        <v>14</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -9910,23 +10185,73 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>20:03</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>54</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>18:51:28</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>20:41</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C56" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D55" t="n">
+      <c r="D56" t="n">
         <v>110</v>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>20:42</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>93</v>
+      </c>
+      <c r="E57" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9956,7 +10281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 18:51:28</t>
+          <t>Última actualización: 19:09:10</t>
         </is>
       </c>
     </row>
@@ -10972,7 +11297,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -10986,7 +11311,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -10997,7 +11322,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -11011,7 +11336,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4623
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E342"/>
+  <dimension ref="A1:E349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:10</t>
+          <t>Última actualización: 19:34:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 337</t>
+          <t>Total filas: 344</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2598,7 +2598,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>07:45:25</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2608,11 +2608,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>101</v>
+        <v>12</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2623,7 +2623,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>07:45:25</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>12</v>
+        <v>101</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -4483,7 +4483,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,7 +8048,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -8058,11 +8058,11 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>7</v>
+        <v>101</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
@@ -8312,7 +8312,7 @@
         </is>
       </c>
       <c r="D319" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
@@ -8323,7 +8323,7 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
@@ -8337,7 +8337,7 @@
         </is>
       </c>
       <c r="D320" t="n">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
@@ -8348,7 +8348,7 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
@@ -8362,7 +8362,7 @@
         </is>
       </c>
       <c r="D321" t="n">
-        <v>34</v>
+        <v>9</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
@@ -8423,12 +8423,12 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:56</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -8437,7 +8437,7 @@
         </is>
       </c>
       <c r="D324" t="n">
-        <v>84</v>
+        <v>22</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
@@ -8448,12 +8448,12 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -8462,7 +8462,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,7 +8473,7 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
@@ -8487,7 +8487,7 @@
         </is>
       </c>
       <c r="D326" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8503,16 +8503,16 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,21 +8523,21 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>54</v>
+        <v>28</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,7 +8548,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
@@ -8562,7 +8562,7 @@
         </is>
       </c>
       <c r="D329" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8598,21 +8598,21 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8628,16 +8628,16 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>91</v>
+        <v>101</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,12 +8673,12 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -8687,7 +8687,7 @@
         </is>
       </c>
       <c r="D334" t="n">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8703,16 +8703,16 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>101</v>
+        <v>51</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8753,16 +8753,16 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,12 +8773,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>93</v>
+        <v>67</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8803,16 +8803,16 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8853,16 +8853,16 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>113</v>
+        <v>101</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,23 +8873,198 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D342" t="n">
+        <v>77</v>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>20:51</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D343" t="n">
+        <v>77</v>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>21:01</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D344" t="n">
+        <v>87</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D345" t="n">
+        <v>88</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
           <t>19:09:10</t>
         </is>
       </c>
-      <c r="B342" t="inlineStr">
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D346" t="n">
+        <v>113</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
         <is>
           <t>21:03</t>
         </is>
       </c>
-      <c r="C342" t="inlineStr">
+      <c r="C347" t="inlineStr">
         <is>
           <t>10_OLMOS</t>
         </is>
       </c>
-      <c r="D342" t="n">
+      <c r="D347" t="n">
         <v>114</v>
       </c>
-      <c r="E342" t="inlineStr">
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D348" t="n">
+        <v>96</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>112</v>
+      </c>
+      <c r="E349" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -8919,7 +9094,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:10</t>
+          <t>Última actualización: 19:34:34</t>
         </is>
       </c>
     </row>
@@ -10185,7 +10360,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -10199,7 +10374,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10210,7 +10385,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -10224,7 +10399,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>110</v>
+        <v>67</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -10268,7 +10443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10281,14 +10456,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:09:10</t>
+          <t>Última actualización: 19:34:34</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 41</t>
+          <t>Total filas: 43</t>
         </is>
       </c>
     </row>
@@ -11297,12 +11472,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -11311,7 +11486,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>53</v>
+        <v>27</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -11327,18 +11502,68 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>20:02</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>53</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>19:34:33</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>67</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D46" t="n">
+      <c r="D48" t="n">
         <v>93</v>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4624
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E349"/>
+  <dimension ref="A1:E356"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:34</t>
+          <t>Última actualización: 19:52:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 344</t>
+          <t>Total filas: 351</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -6258,7 +6258,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>7</v>
+        <v>101</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,7 +8048,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -8058,11 +8058,11 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8448,12 +8448,12 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>19:59</t>
+          <t>19:57</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -8462,7 +8462,7 @@
         </is>
       </c>
       <c r="D325" t="n">
-        <v>84</v>
+        <v>5</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -8473,21 +8473,21 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>20:01</t>
+          <t>19:59</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D326" t="n">
-        <v>27</v>
+        <v>84</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
@@ -8528,16 +8528,16 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>20:02</t>
+          <t>20:01</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8548,21 +8548,21 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
@@ -8573,21 +8573,21 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D330" t="n">
-        <v>54</v>
+        <v>10</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8608,11 +8608,11 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,21 +8623,21 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>100</v>
+        <v>54</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,21 +8648,21 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>101</v>
+        <v>54</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -8673,21 +8673,21 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:04</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D334" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8723,21 +8723,21 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>51</v>
+        <v>101</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,21 +8773,21 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D338" t="n">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>101</v>
+        <v>44</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,21 +8898,21 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D343" t="n">
-        <v>77</v>
+        <v>93</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>87</v>
+        <v>53</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>113</v>
+        <v>77</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,21 +8998,21 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>114</v>
+        <v>59</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9028,16 +9028,16 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,23 +9048,198 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D349" t="n">
+        <v>70</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D350" t="n">
+        <v>70</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>21:02</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D351" t="n">
+        <v>113</v>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>19:09:10</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>21:03</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D352" t="n">
+        <v>114</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D353" t="n">
+        <v>78</v>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr">
+      <c r="C354" t="inlineStr">
         <is>
           <t>11_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D349" t="n">
-        <v>112</v>
-      </c>
-      <c r="E349" t="inlineStr">
+      <c r="D354" t="n">
+        <v>94</v>
+      </c>
+      <c r="E354" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D355" t="n">
+        <v>102</v>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>113</v>
+      </c>
+      <c r="E356" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9081,7 +9256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9094,14 +9269,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:34</t>
+          <t>Última actualización: 19:52:40</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 52</t>
+          <t>Total filas: 53</t>
         </is>
       </c>
     </row>
@@ -10360,12 +10535,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>20:03</t>
+          <t>20:02</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -10374,7 +10549,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -10390,16 +10565,16 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:03</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>67</v>
+        <v>29</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -10410,23 +10585,48 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>19:52:40</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>20:41</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>49</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>19:09:10</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>20:42</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>215B_EL PATO</t>
         </is>
       </c>
-      <c r="D57" t="n">
+      <c r="D58" t="n">
         <v>93</v>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10456,7 +10656,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:34:34</t>
+          <t>Última actualización: 19:52:40</t>
         </is>
       </c>
     </row>
@@ -11472,7 +11672,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -11486,7 +11686,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -11522,7 +11722,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11536,7 +11736,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>67</v>
+        <v>49</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4625
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E356"/>
+  <dimension ref="A1:E361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:40</t>
+          <t>Última actualización: 20:09:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 351</t>
+          <t>Total filas: 356</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2398,7 +2398,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>51</v>
+        <v>17</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2423,7 +2423,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2433,11 +2433,11 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -8023,7 +8023,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>17:35:27</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
@@ -8033,11 +8033,11 @@
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D308" t="n">
-        <v>101</v>
+        <v>7</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
@@ -8048,7 +8048,7 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:35:27</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
@@ -8058,11 +8058,11 @@
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D309" t="n">
-        <v>7</v>
+        <v>101</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8608,11 +8608,11 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8633,11 +8633,11 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8698,21 +8698,21 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>20:10</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D335" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
@@ -8728,16 +8728,16 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>20:16</t>
+          <t>20:15</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D336" t="n">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
@@ -8748,21 +8748,21 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>20:22</t>
+          <t>20:16</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D337" t="n">
-        <v>30</v>
+        <v>101</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
@@ -8773,12 +8773,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>20:23</t>
+          <t>20:22</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -8787,7 +8787,7 @@
         </is>
       </c>
       <c r="D338" t="n">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
@@ -8798,21 +8798,21 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>20:25</t>
+          <t>20:23</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D339" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
@@ -8823,21 +8823,21 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>20:32</t>
+          <t>20:25</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D340" t="n">
-        <v>101</v>
+        <v>16</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
@@ -8848,21 +8848,21 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>20:36</t>
+          <t>20:32</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D341" t="n">
-        <v>44</v>
+        <v>101</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
@@ -8873,21 +8873,21 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>20:41</t>
+          <t>20:36</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D342" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,12 +8898,12 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>20:42</t>
+          <t>20:41</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -8912,7 +8912,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8923,21 +8923,21 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:42</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D344" t="n">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="E344" t="inlineStr">
         <is>
@@ -8948,21 +8948,21 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D345" t="n">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,7 +8998,7 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
@@ -9008,11 +9008,11 @@
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D347" t="n">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9028,16 +9028,16 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9053,16 +9053,16 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>70</v>
+        <v>59</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,21 +9073,21 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>70</v>
+        <v>43</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,21 +9123,21 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D352" t="n">
-        <v>114</v>
+        <v>70</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9153,16 +9153,16 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,21 +9173,21 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>102</v>
+        <v>54</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,23 +9223,148 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>21:10</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D356" t="n">
+        <v>61</v>
+      </c>
+      <c r="E356" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D357" t="n">
+        <v>77</v>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D358" t="n">
+        <v>85</v>
+      </c>
+      <c r="E358" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D359" t="n">
+        <v>87</v>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
           <t>19:52:40</t>
         </is>
       </c>
-      <c r="B356" t="inlineStr">
+      <c r="B360" t="inlineStr">
         <is>
           <t>21:45</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr">
+      <c r="C360" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D356" t="n">
+      <c r="D360" t="n">
         <v>113</v>
       </c>
-      <c r="E356" t="inlineStr">
+      <c r="E360" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>21:46</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>97</v>
+      </c>
+      <c r="E361" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9269,7 +9394,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:40</t>
+          <t>Última actualización: 20:09:04</t>
         </is>
       </c>
     </row>
@@ -10610,7 +10735,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -10624,7 +10749,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -10643,7 +10768,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10656,14 +10781,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 19:52:40</t>
+          <t>Última actualización: 20:09:04</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 43</t>
+          <t>Total filas: 44</t>
         </is>
       </c>
     </row>
@@ -11747,7 +11872,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -11761,9 +11886,34 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>93</v>
+        <v>33</v>
       </c>
       <c r="E48" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>21:26</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>77</v>
+      </c>
+      <c r="E49" t="inlineStr">
         <is>
           <t>L6203</t>
         </is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4626
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E361"/>
+  <dimension ref="A1:E367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:04</t>
+          <t>Última actualización: 20:31:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 356</t>
+          <t>Total filas: 362</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -2858,7 +2858,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D101" t="n">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D102" t="n">
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>94</v>
+        <v>61</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8608,7 +8608,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -8658,7 +8658,7 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D333" t="n">
@@ -8873,7 +8873,7 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
@@ -8887,7 +8887,7 @@
         </is>
       </c>
       <c r="D342" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
@@ -8898,7 +8898,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
@@ -8912,7 +8912,7 @@
         </is>
       </c>
       <c r="D343" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -8948,12 +8948,12 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>20:44</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -8962,7 +8962,7 @@
         </is>
       </c>
       <c r="D345" t="n">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="E345" t="inlineStr">
         <is>
@@ -8973,21 +8973,21 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>20:50</t>
+          <t>20:45</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D346" t="n">
-        <v>101</v>
+        <v>36</v>
       </c>
       <c r="E346" t="inlineStr">
         <is>
@@ -8998,12 +8998,12 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>20:51</t>
+          <t>20:50</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -9012,7 +9012,7 @@
         </is>
       </c>
       <c r="D347" t="n">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="E347" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9062,7 +9062,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9078,16 +9078,16 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>20:52</t>
+          <t>20:51</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9098,21 +9098,21 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:52</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D351" t="n">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="E351" t="inlineStr">
         <is>
@@ -9123,12 +9123,12 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -9137,7 +9137,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,7 +9148,7 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
@@ -9162,7 +9162,7 @@
         </is>
       </c>
       <c r="D353" t="n">
-        <v>70</v>
+        <v>31</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,7 +9173,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -9183,11 +9183,11 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,21 +9198,21 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>54</v>
+        <v>113</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9228,16 +9228,16 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,21 +9248,21 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>77</v>
+        <v>38</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9278,16 +9278,16 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D358" t="n">
-        <v>85</v>
+        <v>61</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,21 +9298,21 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>87</v>
+        <v>55</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>113</v>
+        <v>62</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9353,18 +9353,168 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
+          <t>21:34</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
+        </is>
+      </c>
+      <c r="D361" t="n">
+        <v>85</v>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>21:36</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D362" t="n">
+        <v>65</v>
+      </c>
+      <c r="E362" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>14X44_ABASTO</t>
+        </is>
+      </c>
+      <c r="D363" t="n">
+        <v>74</v>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>20:09:04</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
           <t>21:46</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr">
+      <c r="C364" t="inlineStr">
         <is>
           <t>14X44_ABASTO</t>
         </is>
       </c>
-      <c r="D361" t="n">
+      <c r="D364" t="n">
         <v>97</v>
       </c>
-      <c r="E361" t="inlineStr">
+      <c r="E364" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>22:03</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D365" t="n">
+        <v>92</v>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D366" t="n">
+        <v>100</v>
+      </c>
+      <c r="E366" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>119</v>
+      </c>
+      <c r="E367" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9394,7 +9544,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:04</t>
+          <t>Última actualización: 20:31:44</t>
         </is>
       </c>
     </row>
@@ -10710,7 +10860,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -10724,7 +10874,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -10768,7 +10918,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10781,14 +10931,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:09:04</t>
+          <t>Última actualización: 20:31:44</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 44</t>
+          <t>Total filas: 46</t>
         </is>
       </c>
     </row>
@@ -11847,7 +11997,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:31:44</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -11861,7 +12011,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -11897,25 +12047,75 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>21:25</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>54</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>20:09:04</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>21:26</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>215C_LA PLATA</t>
         </is>
       </c>
-      <c r="D49" t="n">
+      <c r="D50" t="n">
         <v>77</v>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>20:31:44</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-40 Y 115</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>104</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>L6173</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4627
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E367"/>
+  <dimension ref="A1:E371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:44</t>
+          <t>Última actualización: 20:50:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 362</t>
+          <t>Total filas: 366</t>
         </is>
       </c>
     </row>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1433,11 +1433,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1448,7 +1448,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1458,11 +1458,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -3058,11 +3058,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>93</v>
+        <v>58</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -3073,7 +3073,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>26</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -4273,7 +4273,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>14</v>
+        <v>87</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
@@ -4298,7 +4298,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -4308,11 +4308,11 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>87</v>
+        <v>14</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>19</v>
+        <v>94</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>109</v>
+        <v>9</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7523,7 +7523,7 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>16:50:26</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
@@ -7533,11 +7533,11 @@
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D288" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
@@ -7548,7 +7548,7 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>16:50:26</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
@@ -7558,11 +7558,11 @@
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D289" t="n">
-        <v>13</v>
+        <v>93</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -8098,7 +8098,7 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
@@ -8108,11 +8108,11 @@
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D311" t="n">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
@@ -8123,7 +8123,7 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
@@ -8133,11 +8133,11 @@
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D312" t="n">
-        <v>13</v>
+        <v>89</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8508,11 +8508,11 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8533,11 +8533,11 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8608,7 +8608,7 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D331" t="n">
@@ -8623,7 +8623,7 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
@@ -8633,11 +8633,11 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D332" t="n">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -9023,7 +9023,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -9033,11 +9033,11 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>77</v>
+        <v>42</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9062,7 +9062,7 @@
         </is>
       </c>
       <c r="D349" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9073,7 +9073,7 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
@@ -9083,11 +9083,11 @@
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D350" t="n">
-        <v>42</v>
+        <v>77</v>
       </c>
       <c r="E350" t="inlineStr">
         <is>
@@ -9123,12 +9123,12 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>21:01</t>
+          <t>20:56</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -9137,7 +9137,7 @@
         </is>
       </c>
       <c r="D352" t="n">
-        <v>87</v>
+        <v>6</v>
       </c>
       <c r="E352" t="inlineStr">
         <is>
@@ -9148,21 +9148,21 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>21:02</t>
+          <t>21:01</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D353" t="n">
-        <v>31</v>
+        <v>87</v>
       </c>
       <c r="E353" t="inlineStr">
         <is>
@@ -9173,7 +9173,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -9183,11 +9183,11 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,7 +9198,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -9208,11 +9208,11 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>113</v>
+        <v>70</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9223,12 +9223,12 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>21:03</t>
+          <t>21:02</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -9237,7 +9237,7 @@
         </is>
       </c>
       <c r="D356" t="n">
-        <v>54</v>
+        <v>12</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9248,21 +9248,21 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>21:09</t>
+          <t>21:03</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D357" t="n">
-        <v>38</v>
+        <v>54</v>
       </c>
       <c r="E357" t="inlineStr">
         <is>
@@ -9273,12 +9273,12 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>21:10</t>
+          <t>21:09</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -9287,7 +9287,7 @@
         </is>
       </c>
       <c r="D358" t="n">
-        <v>61</v>
+        <v>19</v>
       </c>
       <c r="E358" t="inlineStr">
         <is>
@@ -9298,21 +9298,21 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>21:26</t>
+          <t>21:10</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D359" t="n">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E359" t="inlineStr">
         <is>
@@ -9323,21 +9323,21 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>21:33</t>
+          <t>21:26</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>84_COLONIA URQUIZA-ESC 49</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D360" t="n">
-        <v>62</v>
+        <v>36</v>
       </c>
       <c r="E360" t="inlineStr">
         <is>
@@ -9348,12 +9348,12 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>21:34</t>
+          <t>21:33</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -9362,7 +9362,7 @@
         </is>
       </c>
       <c r="D361" t="n">
-        <v>85</v>
+        <v>43</v>
       </c>
       <c r="E361" t="inlineStr">
         <is>
@@ -9373,21 +9373,21 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>21:36</t>
+          <t>21:34</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D362" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="E362" t="inlineStr">
         <is>
@@ -9398,21 +9398,21 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>74</v>
+        <v>46</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,12 +9423,12 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -9437,7 +9437,7 @@
         </is>
       </c>
       <c r="D364" t="n">
-        <v>97</v>
+        <v>55</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,21 +9448,21 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>22:03</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D365" t="n">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>22:11</t>
+          <t>22:03</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,23 +9498,123 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
+          <t>22:11</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D367" t="n">
+        <v>81</v>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>20:50:48</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="C367" t="inlineStr">
+      <c r="C368" t="inlineStr">
         <is>
           <t>23_HERNANDEZ</t>
         </is>
       </c>
-      <c r="D367" t="n">
-        <v>119</v>
-      </c>
-      <c r="E367" t="inlineStr">
+      <c r="D368" t="n">
+        <v>100</v>
+      </c>
+      <c r="E368" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>20:50:48</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D369" t="n">
+        <v>103</v>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>20:50:48</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D370" t="n">
+        <v>106</v>
+      </c>
+      <c r="E370" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>20:50:48</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>22:43</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>113</v>
+      </c>
+      <c r="E371" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9531,7 +9631,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9544,14 +9644,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:44</t>
+          <t>Última actualización: 20:50:48</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 53</t>
+          <t>Total filas: 54</t>
         </is>
       </c>
     </row>
@@ -10902,6 +11002,31 @@
         <v>33</v>
       </c>
       <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>20:50:48</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>103</v>
+      </c>
+      <c r="E59" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -10931,7 +11056,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:31:44</t>
+          <t>Última actualización: 20:50:48</t>
         </is>
       </c>
     </row>
@@ -12047,7 +12172,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -12061,7 +12186,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -12097,7 +12222,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>20:31:44</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -12111,7 +12236,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4628
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E371"/>
+  <dimension ref="A1:E379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:48</t>
+          <t>Última actualización: 21:34:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 366</t>
+          <t>Total filas: 374</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2173,7 +2173,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:39:26</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>08:39:26</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2208,11 +2208,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2483,7 +2483,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D87" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D192" t="n">
@@ -5158,7 +5158,7 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D193" t="n">
@@ -5858,7 +5858,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6483,7 +6483,7 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D246" t="n">
@@ -6748,7 +6748,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>16:09:25</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -6758,11 +6758,11 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
@@ -6773,7 +6773,7 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>16:09:25</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -6783,11 +6783,11 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D258" t="n">
-        <v>32</v>
+        <v>10</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
@@ -7083,7 +7083,7 @@
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D270" t="n">
@@ -7108,7 +7108,7 @@
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D271" t="n">
@@ -7648,7 +7648,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>18:35:31</t>
+          <t>18:10:26</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D293" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
@@ -7673,7 +7673,7 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>18:10:26</t>
+          <t>18:35:31</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
@@ -7683,11 +7683,11 @@
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D294" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
@@ -7708,7 +7708,7 @@
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>15X38_ABASTO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D295" t="n">
@@ -7733,7 +7733,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>15X38_ABASTO</t>
         </is>
       </c>
       <c r="D296" t="n">
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8508,11 +8508,11 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8533,11 +8533,11 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -9023,7 +9023,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -9033,11 +9033,11 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9173,7 +9173,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -9183,11 +9183,11 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>113</v>
+        <v>12</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9223,7 +9223,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
@@ -9233,11 +9233,11 @@
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D356" t="n">
-        <v>12</v>
+        <v>113</v>
       </c>
       <c r="E356" t="inlineStr">
         <is>
@@ -9398,7 +9398,7 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
@@ -9408,11 +9408,11 @@
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>84_COLONIA URQUIZA-ESC 49</t>
         </is>
       </c>
       <c r="D363" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="E363" t="inlineStr">
         <is>
@@ -9423,21 +9423,21 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>21:36</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>14X44_ABASTO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D364" t="n">
-        <v>55</v>
+        <v>2</v>
       </c>
       <c r="E364" t="inlineStr">
         <is>
@@ -9448,12 +9448,12 @@
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t>21:46</t>
+          <t>21:45</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -9462,7 +9462,7 @@
         </is>
       </c>
       <c r="D365" t="n">
-        <v>97</v>
+        <v>11</v>
       </c>
       <c r="E365" t="inlineStr">
         <is>
@@ -9473,21 +9473,21 @@
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t>22:03</t>
+          <t>21:46</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>14X44_ABASTO</t>
         </is>
       </c>
       <c r="D366" t="n">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="E366" t="inlineStr">
         <is>
@@ -9498,21 +9498,21 @@
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t>22:11</t>
+          <t>21:58</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D367" t="n">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="E367" t="inlineStr">
         <is>
@@ -9528,16 +9528,16 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t>22:30</t>
+          <t>22:03</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D368" t="n">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="E368" t="inlineStr">
         <is>
@@ -9548,21 +9548,21 @@
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t>22:33</t>
+          <t>22:04</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D369" t="n">
-        <v>103</v>
+        <v>30</v>
       </c>
       <c r="E369" t="inlineStr">
         <is>
@@ -9573,21 +9573,21 @@
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t>22:36</t>
+          <t>22:11</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D370" t="n">
-        <v>106</v>
+        <v>37</v>
       </c>
       <c r="E370" t="inlineStr">
         <is>
@@ -9598,23 +9598,223 @@
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>22:29</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D371" t="n">
+        <v>55</v>
+      </c>
+      <c r="E371" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
           <t>20:50:48</t>
         </is>
       </c>
-      <c r="B371" t="inlineStr">
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D372" t="n">
+        <v>100</v>
+      </c>
+      <c r="E372" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D373" t="n">
+        <v>57</v>
+      </c>
+      <c r="E373" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>22:33</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D374" t="n">
+        <v>59</v>
+      </c>
+      <c r="E374" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>22:36</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D375" t="n">
+        <v>62</v>
+      </c>
+      <c r="E375" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>22:37</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D376" t="n">
+        <v>63</v>
+      </c>
+      <c r="E376" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
         <is>
           <t>22:43</t>
         </is>
       </c>
-      <c r="C371" t="inlineStr">
+      <c r="C377" t="inlineStr">
         <is>
           <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
-      <c r="D371" t="n">
-        <v>113</v>
-      </c>
-      <c r="E371" t="inlineStr">
+      <c r="D377" t="n">
+        <v>69</v>
+      </c>
+      <c r="E377" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>23:04</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D378" t="n">
+        <v>90</v>
+      </c>
+      <c r="E378" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>23:19</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D379" t="n">
+        <v>105</v>
+      </c>
+      <c r="E379" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9631,7 +9831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9644,14 +9844,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:48</t>
+          <t>Última actualización: 21:34:39</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 54</t>
+          <t>Total filas: 55</t>
         </is>
       </c>
     </row>
@@ -11010,23 +11210,48 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>21:34:39</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>22:31</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>57</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>21:34:39</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>22:33</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C60" t="inlineStr">
         <is>
           <t>215C_EL PATO</t>
         </is>
       </c>
-      <c r="D59" t="n">
-        <v>103</v>
-      </c>
-      <c r="E59" t="inlineStr">
+      <c r="D60" t="n">
+        <v>59</v>
+      </c>
+      <c r="E60" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11056,7 +11281,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 20:50:48</t>
+          <t>Última actualización: 21:34:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 Horarios actualizados Línea 141 - 4629
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-22.xlsx
+++ b/data/horarios-141-2026-08-22.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E379"/>
+  <dimension ref="A1:E383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:34:39</t>
+          <t>Última actualización: 23:10:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 374</t>
+          <t>Total filas: 378</t>
         </is>
       </c>
     </row>
@@ -798,7 +798,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>03:54:03</t>
+          <t>03:01:03</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -808,11 +808,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>54</v>
+        <v>107</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -823,7 +823,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>03:01:03</t>
+          <t>03:54:03</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -833,11 +833,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>107</v>
+        <v>54</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1373,7 +1373,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>06:59:54</t>
+          <t>06:43:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1383,11 +1383,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>06:43:00</t>
+          <t>06:59:54</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1408,11 +1408,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1608,7 +1608,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -2248,7 +2248,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2273,7 +2273,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2283,11 +2283,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2533,7 +2533,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D88" t="n">
@@ -2558,7 +2558,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D89" t="n">
@@ -2773,7 +2773,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>28</v>
+        <v>82</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2798,7 +2798,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>11_ETCHEVERRY</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>82</v>
+        <v>28</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3133,7 +3133,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D112" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D113" t="n">
@@ -3173,7 +3173,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -3183,11 +3183,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -3198,7 +3198,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -3208,11 +3208,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>72</v>
+        <v>26</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -3223,7 +3223,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>26</v>
+        <v>92</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -3323,7 +3323,7 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>10:00:55</t>
+          <t>10:38:41</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -3333,11 +3333,11 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_P INDUSTRIAL</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -3348,7 +3348,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>10:38:41</t>
+          <t>10:00:55</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -3358,11 +3358,11 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>15_P INDUSTRIAL</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -3473,7 +3473,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -3483,11 +3483,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>2</v>
+        <v>103</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -3498,7 +3498,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -3508,11 +3508,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>103</v>
+        <v>2</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -3523,7 +3523,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>09:14:58</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>81_EL PELIGRO</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>104</v>
+        <v>3</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -3548,7 +3548,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>09:14:58</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -3558,11 +3558,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>81_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>3</v>
+        <v>104</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>10:55:24</t>
+          <t>11:09:57</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -3733,11 +3733,11 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>225_C ROCA-H SUR</t>
         </is>
       </c>
       <c r="D136" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -3748,7 +3748,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>11:09:57</t>
+          <t>10:55:24</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>225_C ROCA-H SUR</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>12:08:56</t>
+          <t>13:09:21</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -4783,11 +4783,11 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>15_ABASTO</t>
         </is>
       </c>
       <c r="D178" t="n">
-        <v>65</v>
+        <v>4</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4798,7 +4798,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>13:09:21</t>
+          <t>12:08:56</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -4808,11 +4808,11 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>15_ABASTO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D179" t="n">
-        <v>4</v>
+        <v>65</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
@@ -5683,11 +5683,11 @@
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>11X44_ETCHEVERRY</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D214" t="n">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
@@ -5698,7 +5698,7 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>13:36:29</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
@@ -5708,11 +5708,11 @@
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>11X44_ETCHEVERRY</t>
         </is>
       </c>
       <c r="D215" t="n">
-        <v>94</v>
+        <v>19</v>
       </c>
       <c r="E215" t="inlineStr">
         <is>
@@ -5723,7 +5723,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>13:36:29</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -5733,11 +5733,11 @@
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D216" t="n">
-        <v>61</v>
+        <v>94</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
@@ -5998,7 +5998,7 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:33:10</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
@@ -6008,11 +6008,11 @@
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D227" t="n">
-        <v>16</v>
+        <v>54</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
@@ -6023,7 +6023,7 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>14:33:10</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
@@ -6033,11 +6033,11 @@
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D228" t="n">
-        <v>54</v>
+        <v>16</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
@@ -6433,7 +6433,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>17X38_ROMERO</t>
         </is>
       </c>
       <c r="D244" t="n">
@@ -6448,7 +6448,7 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>14:09:59</t>
+          <t>15:11:48</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
@@ -6458,11 +6458,11 @@
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D245" t="n">
-        <v>118</v>
+        <v>56</v>
       </c>
       <c r="E245" t="inlineStr">
         <is>
@@ -6473,7 +6473,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>15:11:48</t>
+          <t>14:09:59</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -6483,11 +6483,11 @@
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>17X38_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D246" t="n">
-        <v>56</v>
+        <v>118</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
@@ -6698,7 +6698,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>14:51:51</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -6708,11 +6708,11 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>16_P MOR-SANTA ANA</t>
+          <t>225_GOMEZ</t>
         </is>
       </c>
       <c r="D255" t="n">
-        <v>9</v>
+        <v>109</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>14:51:51</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -6733,11 +6733,11 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>225_GOMEZ</t>
+          <t>16_P MOR-SANTA ANA</t>
         </is>
       </c>
       <c r="D256" t="n">
-        <v>109</v>
+        <v>9</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
@@ -7298,7 +7298,7 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>17:53:20</t>
+          <t>16:31:31</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
@@ -7308,11 +7308,11 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>215_EL PELIGRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D279" t="n">
-        <v>0</v>
+        <v>82</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
@@ -7323,7 +7323,7 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>16:31:31</t>
+          <t>17:53:20</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
@@ -7333,11 +7333,11 @@
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>215_EL PELIGRO</t>
         </is>
       </c>
       <c r="D280" t="n">
-        <v>82</v>
+        <v>0</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
@@ -7783,7 +7783,7 @@
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>17_ROMERO</t>
         </is>
       </c>
       <c r="D298" t="n">
@@ -7808,7 +7808,7 @@
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>17_ROMERO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D299" t="n">
@@ -8498,7 +8498,7 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>18:51:28</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
@@ -8508,11 +8508,11 @@
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D327" t="n">
-        <v>70</v>
+        <v>27</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
@@ -8523,7 +8523,7 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>18:51:28</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
@@ -8533,11 +8533,11 @@
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D328" t="n">
-        <v>27</v>
+        <v>70</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -8558,7 +8558,7 @@
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D329" t="n">
@@ -8583,7 +8583,7 @@
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D330" t="n">
@@ -8598,7 +8598,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>19:09:10</t>
+          <t>19:34:33</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
@@ -8608,11 +8608,11 @@
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>14_ABASTO</t>
+          <t>215C_EL PATO</t>
         </is>
       </c>
       <c r="D331" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
@@ -8633,7 +8633,7 @@
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>16_SANTA ANA</t>
+          <t>14_ABASTO</t>
         </is>
       </c>
       <c r="D332" t="n">
@@ -8648,7 +8648,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>19:34:33</t>
+          <t>19:09:10</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
@@ -8658,11 +8658,11 @@
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>215C_EL PATO</t>
+          <t>16_SANTA ANA</t>
         </is>
       </c>
       <c r="D333" t="n">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
@@ -9023,7 +9023,7 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>20:09:04</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
@@ -9033,11 +9033,11 @@
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>23_HERNANDEZ</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D348" t="n">
-        <v>1</v>
+        <v>42</v>
       </c>
       <c r="E348" t="inlineStr">
         <is>
@@ -9048,7 +9048,7 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>20:09:04</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
@@ -9058,11 +9058,11 @@
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>23_HERNANDEZ</t>
         </is>
       </c>
       <c r="D349" t="n">
-        <v>42</v>
+        <v>1</v>
       </c>
       <c r="E349" t="inlineStr">
         <is>
@@ -9173,7 +9173,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>20:50:48</t>
+          <t>19:52:40</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
@@ -9183,11 +9183,11 @@
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>10_OLMOS</t>
+          <t>27_EL RETIRO</t>
         </is>
       </c>
       <c r="D354" t="n">
-        <v>12</v>
+        <v>70</v>
       </c>
       <c r="E354" t="inlineStr">
         <is>
@@ -9198,7 +9198,7 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>19:52:40</t>
+          <t>20:50:48</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
@@ -9208,11 +9208,11 @@
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>27_EL RETIRO</t>
+          <t>10_OLMOS</t>
         </is>
       </c>
       <c r="D355" t="n">
-        <v>70</v>
+        <v>12</v>
       </c>
       <c r="E355" t="inlineStr">
         <is>
@@ -9798,7 +9798,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>21:34:39</t>
+          <t>23:10:47</t>
         </is>
       </c>
       <c r="B379" t="inlineStr">
@@ -9812,9 +9812,109 @@
         </is>
       </c>
       <c r="D379" t="n">
-        <v>105</v>
+        <v>9</v>
       </c>
       <c r="E379" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>23:10:47</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>23:34</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D380" t="n">
+        <v>24</v>
+      </c>
+      <c r="E380" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>23:10:47</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D381" t="n">
+        <v>29</v>
+      </c>
+      <c r="E381" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>23:10:47</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>23:46</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D382" t="n">
+        <v>36</v>
+      </c>
+      <c r="E382" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>23:10:47</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>23:58</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D383" t="n">
+        <v>48</v>
+      </c>
+      <c r="E383" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -9831,7 +9931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E60"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9844,14 +9944,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:34:39</t>
+          <t>Última actualización: 23:10:47</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 55</t>
+          <t>Total filas: 56</t>
         </is>
       </c>
     </row>
@@ -10310,7 +10410,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08:20:07</t>
+          <t>08:54:24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -10320,11 +10420,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>215A_EL PATO</t>
+          <t>215B_EL PATO</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -10335,7 +10435,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08:54:24</t>
+          <t>08:20:07</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -10345,11 +10445,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>215B_EL PATO</t>
+          <t>215A_EL PATO</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1</v>
+        <v>35</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -11252,6 +11352,31 @@
         <v>59</v>
       </c>
       <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>23:10:47</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>23:39</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>29</v>
+      </c>
+      <c r="E61" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -11281,7 +11406,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 21:34:39</t>
+          <t>Última actualización: 23:10:47</t>
         </is>
       </c>
     </row>

</xml_diff>